<commit_message>
Finalizando tela de Clientes e finalizando projeto.
</commit_message>
<xml_diff>
--- a/Fotos Produtos.xlsx
+++ b/Fotos Produtos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f94f6b2d1d795029/Desktop/Daniel/BIs para portifólio/Vendas/Analise_De_Vendas_PowerBI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{99F7304B-343B-4B7D-93D1-37B38071A7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1924AD0E-DD27-4FC6-B7DB-F6107F865FC7}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{99F7304B-343B-4B7D-93D1-37B38071A7EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41107C85-8DD2-4759-A4B5-8D4F41E7F3ED}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{11C8409F-65C0-4867-8478-8012E7136587}"/>
   </bookViews>
@@ -158,9 +158,6 @@
     <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/2wCEAAkGBxMTEhISEhIWFhUVFRYZFhUSFRgWGhgYGhcXFxcYFRgaHSggGholHxcVITEhJiorLi4uFx8zODMtNygtLisBCgoKDg0OGxAQGy4lHyUuLS82MS8tLS0tMy0tLS0wLSstLy0tKy0rNy0vNy0tLS8tLS0tLi0tLS0tLS0tLystLf/AABEIAOAA4QMBIgACEQEDEQH/xAAcAAEAAgMBAQEAAAAAAAAAAAAABgcEBQgDAgH/xABOEAABAwEEBQUJDAcHBQAAAAABAAIRAwQSITEFBkFRYQcTIoGRFCMyUnGhscHRJDM1QmJyc3SSsrPwFSU0Q1OCowhjotLT4fEWF0STw//EABoBAQEAAwEBAAAAAAAAAAAAAAABAgMEBQb/xAAxEQEAAgECAwUHAgcAAAAAAAAAAQIDBBEhMUESMlFhsRMUcYGRofAFIyIkM8HR4fH/2gAMAwEAAhEDEQA/ALxREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEXjaq11sgTitDbdbqdJ7qb2uvNAJusc6BEySBksq1m3CIY2vWsb2nZJEUYsWuFOo+5gC6SzE4tAmXYC6c+iccFl6P1gFZl+m0lskSQRMZxOYSaWjnCVyUtwiYbxFrf0i7xUGkH+IsWbZIsKjaKjsmgcTIXzVtdRpgs7EGeihmtOttazOphlNhvBxN8O2EZQ4b1jjWm34g2eiIJEuJaDBYMCXQZNRgB4rdGC0xFvFz21NK2mvHh5J2ig1PWm3H/AMWnkDiSM3FoGecg4cF5WTXW11GhzbKwguLR0iJcGOeQBtwaevBX3e/l9U96p5/SU+RQbR+u9Z9obQdQYJcWkteTBAJMbDlCm1J8tB3ha747Unazbjy1yRvV9oiLBsEREBERAREQEREBERAREQEREHhbXgNk5SFDbRZucttU3n02Oogc4wCHeACySI39ikGthd3OWsddL3NaSNxz9CjbtWKpAIquI4OKzpeab7NWXFGSIiek7tXT0Y57nUQy6wVHkVHgjotF1oB+Vhl5dilGr9tHMMa+mabmdEtIgGMnN3z6ZWkdq9UGb3/aK8n6EcPjv+0fas8mebxtLXh0tcVu1EpgbXT3helLSdNs4jtUCtGjXAYOef5j7VhO0U45vf8AaPtXPNnXFd1ku0/S/JC/P+oKf5IVbjRzRm532ne1fjrE3e6fnFY9pl2IbbX7SlJ7qRwwa/bxavU1iHCXTfqhplgdF9xAfBEBt6gw7hMjjBtPaOBLMTkfjE7lrP0Z8p32jsyXrYazfFX5+rw9RNaZ7+e3os6naXltMU6l4Pa5wvRsuuBOeJJYMceltGKxdEWiabQx91vSIZekiHc2Ybn+8cfLG2FXX6HJwvO7Sv0aCfsc77RWz2U7bNftqb77z9fgnlgtLBb2XiJvycIxLL2I2OxxG+VaVAy1pGUBc/6H1fe2vRcKhBvHafFcr50VXc+jSe6LzmNLoykjGFx6vvRHk7tB2exaazzllIiwaelqLqxoNeDUaCXNAOERMmI+MO1ckzEc3czkXzeXh3fT5w0r3TABuwcjljkpNojnJsyURFkCLBOl6PPdz3xzviAGR0S/ExAwBKzLynag2fSLGfb6YqCkXQ8gODYORN0Gcs8FkpFonkbCIioIiICIiDS62HvAO6oz0x618aItYIuyO3JeutrfctTgaZ/qNVTaD19YHPqcy+KhDgA9oIFxjcePR86kzPQXDUxWC+nPHyb1rdWdPC0UXkMLeaiZIMyCcOxaSx67sbeJov6br4h7RmG8M8FjvPgqQVKIMgcMe1eBsrRsnyry1c0iLQxxDS25daZIM9EGR2rPqsT4soaLSLulAGwYBa02Oq5xIgDDwvZmt/aXAZkDzLEZUBMA/ny5KbMkb07ZS005IJIdl1L2pmlEYYRjzABMZY3uAny7cV7ayt6VLyO9IWJZA2Ok1xPyXgbuB4r2NPH7Nfzq+e1lttRb5ejPDqePg5xhQGW/PA4nsXuKtPe3MfuBsjj5lit5vxXx88ceHkX6404MNdOwl4jIZiN87Vs7P5wcs3ny+7BFWLTSAyvHZHxXK2dBj3PQ+jZ90Kk2VvdNL5x+65XfohsUKI3UmfdC4tZ34+D1v06NsU/H/DLVfaNc4aVtrmNvODKt1sxedFKBOyThKzeVDW6to6jQfQZTc6rVuHnQ4gC6XSA0jHDeqrsuvdsp2mpamso36k3gWPu9K5MC/PxBt3rzc1Jt2dukvSrOy8jXrCiXiiDXuNJpXhF7dfywx2rW0CTpAlwg8xSkTMGRInaqz/7tW+ferN/66n+qsRvKTbefNo5uz3i0NIuVIgYiO+TPWtd8VrdnyndlE7br/RRXk31mq6Qsrq9ZjGvbWfTinIaQ0NIMOJI8LfsXzyl6z1dH2RteixjnuqsZFW8WgEOJMNIJ8HftXW1taZ/TdSBJDWkDKT3M/D0KUULRWNG+6iBX5tx5q8CJBNwX8sfLhKo0a92wWp1suUecMS24+5gwsyvzkd+a2h5WdITPNWbL+HU/1Vy1x2iZ85mWcysd73ut1A1G3XGzMLmgzddzwkTtzUtXP9TlItrq7a5p2e81gZAZUuwHX/4kzPFWbyZa21tIUq7q7KbXUqoYOavAEFodiHEwcd6ywY5rNpnrJad9kzREXQwEREBERBrdY2TZa/BhP2el6lzHo84NwIwyOJHAnDEZLqTSlO9RrN303jtaQuX7aXU7RWY6Jvufnseb48zggtzkzM2e04E9IZbRzeQ45/aChVOYbhsGzLgrF5M6DmWGmXiOcJqNEg9FwF2Y3gT1qvNLPdRr2ik+LzHuJg53jeEeUOCCd6ge9VsP3me/oMWVrDaHtBumMW7JzOOaap03UrHSvjFwL4kHovcXDEcCF7aV0e6riHQ03TF2csfGCjJX+l7ZVJcOcfmcA4gdgWbqKD305mdvkC2Fv1Ue4k38/kD/ADrJ1b0G6z3w43r2OQHDeViz3YmsJJdSnc70hY9mrAR3thwzcDvJ38fMFsdZ6YDqUDY70ha2i3ESYxz3cV7Omj9mPzq+Y11pjUW28vSGULSP4dPsO4jfx8y+bVbQGnvVPsd/mUuZb30nVKDbIRTaQGOIMObDwXPIBDiSwnfBGElQ/XWk2lWqMZkIMDZLQSBwkqYssZJ5fdc+mth2/i38eH5uidKr7op/OP3XLoWyshjBuaB2Bc4WUzaaQ3uI7QV0ouTV9/5PV0MbY/mqn+0Ae8WH6z/83Kqqjszu/wBlcnLrRp9wMqPeA+nWbzTD+8Lui5oG8NJdPySqWLjA8mPmXJLtgv78OG3b+epezM/zwXgCd3nC9QYBMdSiro5C/g+p9aq/dpry5e/g6n9ap/cqrZcjtmazRlJzXh/OufUdHxXGA5h4gtXzyzUKbtGVH1HhppPY+mD8epi0MjbIc7yROxVio6o7M7h6pXjf37pjrzX41xutwxjHeknd5woye1PZx9itrkFHeLb9ZA/pM9qqRm0x1K6OQ+zNFgfVa8OdWrPc9o+I5sMDTuMNafIQdqsJKxERFUEREBERB+PEgjeFzVpvQxda6PfP2osb4Pge909/S37F0suf9Kn3do4f3rfxWILZ1dsnM0KNGb3N02MvRE3WgTGyYyUA1w1fLtItbzn7VjJZ73jdynpeDwVkWHJRPWV06UsPBo++5RW7qMuUqdNpm4xrJiJugCY6l7McIAz/ADxC9bZSwkDbs9ixKDJDoPDFY8d9mfDbd6vptO0r0Ywbl4ts7t47T7F9hjv+CpO6xsj+tzRepRud6WrTUQJEzG2M+pbjWd0up8A70hammBhOW2N21e1pf6MfnV8t+oT/ADNvl6Qkdi0tXFOGc85gEB/NB10D5WWHFQnWKsCZlxJxJdmSc1anP2gWhlOlSZ3JzMioHYh/xWhsjoxdxy6RxEY1nygXBaqwZESJjK9AvR1z1ytenyRa07Rs6tTgtStZm2/T/iK6HxttmG+q0dpXSq5o1fPu+yfT0/vLpdc2q770NJ3FWcvlnc6hY3AYNruk7ASzog7pgqo3CQDBjhPqXR3KGWjRluL23gLPVIHyrpuHqdBngubbG83RP5xXLLrh9XR8rsd7V6twHtn1r6c9YduqQx3AY+Taoq9uRBkaOJgw60VSJESOjB8y8OXezufo+ldGDbSwuO4c3VEncJIHWp7oqzsp0aTKTbrGsaGiIwj0rw1judyWk1G3mCjULm7wGEkeZZMXMJEgYHjngdowXzdHyv8AF7V5aOebgvGTt8qzC9YsnzTyyPXOParf5Bme5bW6MHWolpiJHNUhI65VM2p5uujODC6a1NoU2WGyCk2GGhScMIJvMa6TxMqwktyiIqgiIgIiIBK55tj5t2jfntP9RpV/aRq3KVV/i03nsaSueaVhqPovtFoe3vdPosaBhOQndJG/yrOtYnnOzC9pjlG636GnLOwQ6s2dzZeeu7MKN6XtjKlvs1oYZp02w4kEHNxwG3MKubFbKhpscXFvfbpu9HAhhGXAlfVGpUio0vdIIzcdxB277qz/AGo6TLVMZ561j5TP94XYzT9ndAvx85rgO2F7Oe1wvMcHN3tIKg3JrUZUe+nVaH32AtvyYLTiG7RIcDh4vBTK0assm9Rc6k7gXEefHzp2cczwmY+6drPXnEW+HCfvvH3fblj1apBAG0+bMrCr1a1AgVm4bHgSD6PV5CvGnpmmSPCJktAGOMScMDk3MrG9ezz5ePRtxZYycK8/Dr9GHp0zUHAR6Fg0gJEmBvifQvS2Wi+4y0ggnPbO7gvJoxEmBtO7ivS00xOKJh8/r4mNTaJ8vSG3paRDGlja1QMiIa52GeM3cNmAhQzWe5fNwyI2zhvzzVuBz6Z5qnQHNi8AQDBAYHCdhJJIk5wqt1/s7adpqtZg3AwNhLQSB1lYYckWtMRHm6cuG1IiZnfjtymNvhx5Ixq5+32T6en94Lphcz6t/t9k+np/eC6YXLqe+9HSdxo9eLG+to+2UqYl76FQNAzJumAOK5bNoLDduuwJzEbdy7AXMfK08nS1r6TcHMAG6KVPPjMnrXLLqaNtc3ZDZ4SJXkyoa00mMcXvF1oAmXHADtXwyoQwQ5oO85KzP7PtObTaXG6YpCDGIJeMupRV4Wdl1jW7mgdgWJp+zOqWW002iXPo1WtHFzHAecrPRZI5AfUdTJY5jgWkgyIM7QQvanXJEhvVIlSzlvfOlHi80XadIR/LOPaoXReQzwmgzmcvQsVejbVfJaGOJIIAAkzGAjyrqzVyzGnZLLTcIcyhSa4bi2m0EeZUdyDsvaQeTdcBQeZiYdfpgEdpXQSsIIiKgiIgIiINVrVUu2O1H+4qedpA9K511h0gQ1tnDQAbr3EdYA9fYr+5QKt2wWg7wxv2qjG+tc0Wx0134R0o7AG+pXoiTDRzu5WPuXRUpNe0kzJpk0ahG6e9GNxC/KxxZV+LUb0uByf2OF7yFqsjQ+rgfomzNAF8MdUB2kVJvDyQQQN7GqvKNKC+g/DEls7HZEHgYg+QHYivXRFudZ6zXAgFrrzTmJ2jiCCRxDldmgtMU7VTv0w2RF9hPSYeO8bjkVRVz92/AjAE4ZbOBH+25etkt9Si4EOc0jJ7SQfIeHAoL9rU2uBa5jSDgQQfYoVpvQIouFQXjTkdJpIfTOQx2jE574O8x6z8odqaILaNT5TmXT13SAtdpfXa1Vmlpeyk05ik0AngSZPn6lspfbhPJoy4e1xjhaOUpTpge9mZkEzGeSwrNTaTDnXRvWFo7SHPUmnK7ILTsJiY4HPrXuV6eGsRjiKvn9Vkm2ebWjj4fJIaGl3sYGC0YAYGGkgDCASN2UyoTrbSaDeFS+XHGTJxkknzdpWzcVptPtloKsY4rxhlXPN5iJ9ZaHV0+7rL9PT+8umlzBod0Wugd1QHsxXT68/U997el7guXeUp5dpO2YNPfnDGdkN38F1EofytUwdFWskCYp4xj77TC5pdTm5jSWQGtJGw5bcc1an9npnfbY6B73TF4H5TsI6lBNSbGx1vsTXNDgbTTDg4AgicQQcwuoLJYaVKeapMZOfNsa2YymApCshERVHNfLA8u0rasGkDmwJ4UaeeO+VEqLTdIDWk+Ls2cV07yjUwdGW8kAnuarBI+QVzdoOytNpswIBBtNBpBEgg1WAgjcQoqdcgNObdWddHRs7xeBympSwjq8yvtY1k0fRpY0qVNhIg82xrcN2AWSqgiIgIiICIiCK8pj4sLxvqUh/jB9ShOq+g21XtBgjDBwBEKYcqjwLCSSAOdp4kxvUH1OqOmq9tTogw2HiPCGWO6UkiVuUrOGgNaGgAAABsAAYAATgFWHKZq46m8WmmOg49KB4LvYfTKlNHSJvUpqYXm3peMr2M47ltbZpCzOa5j303NcIILwqnCFKC7Vb0sCBnEx84DEt3OEkZGRC8qlF7AJAew5OmQfI8SD1+ZbnWPV00337JUFQYkNa4F7dpwGYicQoz+lLpN4Ppu2uom7Pzm4A+ZFfTwzxT1f8AKUqc+Azrz9vpC8aulJytA/npCe0NPpXkyo6p+9c+NjGvMdoACDfaGrinUAc7F8NI47PPh1nFS/RthNao2mCATOJ2QCfUq8s4YxwDe+VDkymQ+DsvObLR/KXHyKe6t6TbRtLDWNyLwdtuktIjDiu7TXn2dojnHJ5GuwVnNS08p4S2do0C1pcDXktJBDaLyRDQ5xw2AEY8VqtatAmjTbLw8PBggEZAH1qQ2jSlB7nO5+mC4mS17wbpY1hHgbQ1sjsKwNbdKUqrKLab2uLb03JgCGgYkcFspfJNoid/Pg1ZMOGtLTG28cuM+PxVVZW9/Z5T90rp2zVbzGuGTmg9olc4VKN21M3Xif8ACVf2q1W9Y7Mf7lnYGgBcuqja70dHO+PdtVEOVp0aKtXlojtr0lL1DeV8/qm0+Wh+PSXM61Jag/CNi+st9ZXT65i5PR+srF9ZHmY4rp1SAREVEc5RT+rLd9A/ziFzpoD9rsv1yzfjMXRXKQf1XbvoXLnfVse7bJ9dsv4zFFdWIiKoIiICIiAiIghXK7ZH1dHllNpc7nqRgAnAOk4BRjQN6nQZTNOm0gQZpVAcokm5nxVs1aYcIIkLx7iZ4qsSk1iVelzsYFHrZU9beCxqtCoYxo4GfBfjjMHo4jgrL7iZ4qdxM8VN2PYhXWjDUp1b7hRLS26QxrgRjIIluew8ANy/dLaPs1o98otJ8YC6e0ZqxO4meKncTPFRlEbKXtGoFlcZa+o3hIPqX5Q5PbKPCqVHcJaB6FdPcTPFTuFm5RVI6eslKzGk2g24C10lsycRmTitK7Sl1xkTPjAnYr60lq3Qrlpe09EECDGfUvOwaq2ak5zmskuABvw7LdIXZj1FaU26vNyaXJfNNun+vBRf/UAmebHUxfbtZgRHNRxDDKv79EUP4TPst9ifoij/AAmfZb7Fl755L7h5ueqNuFatTDWOJk4XT4rlfWptMtsNka4EEUaYIOBBujArNZouiDIptB3hoHqWW1oAgZBc2bL7S27qwYfZV7L9UL5Yvgq0fPofj01NFCuWH4LrfPo/isWpvUzycidJ2H6w7zU3ldNrmTkz+FLB9M/8Goum1IBERURjlMP6rtv0XrC591VbNusf12y+aswroHlO+C7Z9GPvtVAam/t9i+uUPxGqK6nREVQREQEREBERAREQEREBERAREQEREBERAREQFD+VeiX6OqNG2pS++D6lMFr9N2EVqVw+MD2IKP5O9DObpCxvIwa95/pPHrXQC0OjNAMpvY8DFs+gj1rfICIiCL8pjZ0ZagNrWD+qxUnqZoxwt1jdGVppHseF0HrBY+es9Sn413zOafUtBonVVtN9N8eC8O7DKgmCIioIiICIiAiIgIiICIiAiIgIiICIiAiIgIiICIiAiIgIiICIiAiIgIiICIiAiIgIiICIiAiIgIiICIiAiIgIiICIiAiIgIiICIiAiIgIiICIiD//2Q==</t>
   </si>
   <si>
-    <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/2wCEAAkGBxMTEhUTExMVFRUXFRUYFRcXFxcVGhgVGBgXFxUXFRgYHSggGRolHRcVITEhJSkrLi4uFx8zODMtNygtLisBCgoKDg0OGhAQGy0lICUtLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLS0tLf/AABEIAOEA4QMBEQACEQEDEQH/xAAcAAACAgMBAQAAAAAAAAAAAAADBAIFAAEGBwj/xABMEAACAQIDBAYGBQgHBwUBAAABAhEAAwQSIQUxQVETImFxgZEGMqGxwfAUQlJi0QcVU3KCkrLhIyQzosLT8RZzdJOjs9JDVGODhDT/xAAbAQACAwEBAQAAAAAAAAAAAAADBAABAgUGB//EADsRAAIBAgQCBwYGAQMFAQAAAAABAgMRBBIhMUFRBRMiYXGBkTKhscHR8BQjM0JS4ZIV0vFDU3LC4jT/2gAMAwEAAhEDEQA/APFcIOt4UWG5unudj+TggbSw08S487b0zT4+AHpCN6D8V8T32zhssxGpmfDSsynexwKWGyKVraslYtHiOOtVKSN0qc+KJZY3/wClZvc1lcGnL/gKtvlGvGsth400lpx4ng35W7RG0rk8bdo/3Y+Fbdnax0cBFqm83NnFFazxG5rssewiaCuzhdIo41V6jyJpXXhLsizkPbLTr+B94okJagMQ+wdDhhWZnKldhdvp/VLn7H8a0jVeg3gYZakfvged7RX1+4+9a5uIWkvvkd+k/Z8irUUnbQZZjLxqiIxa3YjDI1U0ZGcMJBq4ogUpWzJgWoRhVWoUwyLVlJBGGlMUeIGvwK+x/bHx+FKVP1WOUv0kPpeZGDKSrAyCDBB5g1RGK3m51GQUeslkIqiwGDiaXp7h6XtHWegWm0cKf/l96sKZhx8H8CsYvyX5fE+gyx3Ad9C0OG27JJHJ+k3p4mDv9C9pmIVWkRHWmN5HKtxjBrVsbo4WtUjnjbzb+hVH8rFk78Pc7dV/GtdXT5v0/sNLo+s/4+r+hNvytWBEYe6eeqD41nq4X1b9P7LWBr2t2V5v6HnnpxtxcbijfRGQdGiwxBMrOunfWWktEPUKMqcbPe/A54rVLc3NdljuEXQfPGuxh9keeqvUfVa6MZaCzY5s1Ot4H4USm9QGIfYOhwa0OtXpx7Lkk/FC9LD1ZdpRdvBhdticNcA10X+JaUnUjJaNDeHpyjUV0/Q852mNX7m/w0rX2Z1aX7fIqrazSEnZDVgrYVyYCmsKtDmaUHyBoI0NGvfYyyTKKiZQXBqQ4q9CFg61owyMVRCairKHcDi2tMHQgEcwD7DQq1CFaGSewSlUlTd0DJ+fOnqC3FMQ9ittGLx8fhSlT9VjlH9JDFxqogC4aogKKohrLUIJYD1/A0CG41R9o670KaNoYQ//ADoPPT40ePyfwNYxfky8vifRSrS12ceMUzxb8r9uMeO2xbP964PhRI6nZwMfyvN/I4iKseymgKhMpmWssy4mitSO4KpHsPwHMKug8ffXYo+yjy9b2h1F0pyL0FW9Ri1c6NS43nqp+sePgPaRSOPxbpRyQ9p+5feg7gsMql6k1otlzf0W78lxC4jElQEnX6x5njNcA6zdxb6SedQgtjrAuqRuYgwY99GhWlFW4GHBN3OdwuKe3osTxkA7uGtEqUY1EsxcZON7D2L27fds2YKd/UVVG6NwFL08BQirW9WbdWb4lapkyaetZWBWuW2Gx9oYV7DWpuG6HS7OoXLlKEct5pOdGo8RGqpdlKzXzNprI4s3h8NbItlX65eGU8uBFbVWoqrUo9m2jKyq2m4e/bIMHeKcTuroDJai5FQhsVCWJqatFWCA01h+IvieBWn+2Pj8KTqfqsbpfpRC3KosGRWSBLVvXUxW4RTkk3Yg79BT9KvlXR/BUv8AuI1pzOe2f647jXDhuM0PbR1fomv9ewmsf1iz/GKZjv6/ANjI/kS8vifRttTJk6eFKNnEhFp6s8d/LIv9eT/h0/7l2iQ2O7gI3peb+RwUVsfUDAKheQ2BQ2ZcDCtXHdAasew/BjmGGgrsUvZR47Ee2x62ulMp6CknqZdabgHC2uv6x1PjML+zXmq9Xrakp+ngtvr5npYUuppxpcUtfF6v00XkK3HkkmhFmgahCYqEKTbVnLcDgaNr4jfTNOWaNjLWoOztUrcLqiaiMpEjXfQ5YVTp5JN+JtVLO6QujSZpq1lYwXOzbGEZb5uuysLLGwACM1/TKCQDp62+KRqzxKlBQWmbteBtRjrcVtYYhxxgjWnISvbQG42HrtHQNgGqiM0KhRNDFXa5adgiU1h1uK4l6ISt5ReOYEjraAxwFJ103Vdhyg11UbhboHARVJMttEAtSxQW2lWkQNkHIVMpRz2A9ceNKw3HcP8AqI6f0cYjGYUjT+s2P+4tMQ3HMVH8mXgfS4HOkbnES5nj/wCWlIxVk87A9lx/xo1J6Hd6Nj+U7c38EeeRRDpKBgFQvISih7lOmTy1a3QvWh2JeDG8Ounia7NH2UeExX6jHrRCgsdy6ntjcPE6eNDxtXq6Dtu9F5/1qXgKSqYiN9l2n4L6uy8xS2jFR9Z7jT2nX4ma4KVjuNtu7G/zQVE3LltB2tJ/D21CgWIwJXLDB1cgKRpqYgEHdvqEGG2NcG4oTyDa+0CoQqdsYNjbZWBDL1hPZvjnIolOVpFM5e3E67uymyiVurJYNbc69nhVWRV2WOzLmjd4+NbiiXGbjVowwJNZISUVaKZNVrSRQULTeHW4tidkVtxoukx9r4UlX0qscofpI02IoeYuxsX6mcliSYmrUyWN/ThzHmKvrDWUqsCeuPGl4bjWF/VR0uwFH0rDzu+kWZ/5i0xHc6GLX5E/A+llw6j6o8qSc2cBQXI8n/LTa/rFgxvtMPJz+Nbpu56Lopfkv/y+SPPMtEudXIbCVlsvKbZapEUQqWdCTyqJ6oXrr8uXgxnB2yYHafIaknsrswnGFPNJ6I+e16cqlbJBXbC7QIVQusMesRHCDljeN4Plu48fF4lV5K2y+7nUw2F/D02923ZvhprZfF7bIJg7yqXucLSQv6zSF9gbzpZBG7IrMfjrmgDb5JO88Nx4cd1akZiWeJfJZsCdczOe9WFYNFl083nWEkHSQ3tgiT41q2lyr62B46XRs0Er1xAC9XdcAA3AaHxrJZ5/jcKbbleE9U8xTsJXVymCQVtlph1mD4+zfWGyDGzXEN4fGiRuZ0Gi1buZZiDUTESJkkDfxK6iqavoU3lVyxuWsxOW0A6iWTmInMANDprK6RqVA1rcouL7RvA1YRlolOL/AGys2v8Axl8n7yz2Pg8JioRiLFzcGiUJO4Os9U9op2nWglmUFLusrnUxODp1YdZQW262a8hb0j9C7tg/0isoPquhLI3cfgYNMOhhMar0nll3aeq+aOK24nLnZ/RmbmcpzQAnxzbvI1xsVga9B9rbnwKVbOrQ37zo9iWdn3IAtszfezufJYX2UFdHuorqsl4K3xRy8VLHR2aS8vqdANgYVtBZUfsR7TWH0XNf9X3nOeLxkd5++5z/AKQbAt4Z7Vy3AzORrDr6rHUDXhw1G8a1qOHySSlK9zqdHY+rVzKXBG/zhe+3Z/55/wDOnPw9T+Xw+o1eh/216P6nHYH1x4+6kYbnawv6qOi2UwW9aYmAt22SeQDAmjp6nYrU3KlJLkfQreleBj/+ux4XFJ8ppNQdzhrC12rKD9Dzn8q+0rOIfDmzdS5lW4GymYkrE+2txTR3uiqE4U5Katrx8DhAlauddQJBao1kJItQHKIyq9U91ZW6FqsOw/Bhtnr1T95sp/VUZ3Htt+BNFxVXM401stX48DyNKkoRnV4vsrw3frovC5B2BspPrNcdj2yrfBV8q5sZN1n4HVqUVHo6EuLlf1TXwSFb2ZEQqYBJYkHQMCQPIAUe100cqMnGSlyJKnSDOqgsBJA0kb5QD+EeA4AMKutpD9bA3j1lFacV819PQlg7F3Fulm2j3HMhFWBodSSYgDtJgc6OcxO52eK9AcWo6ZLtm7cIlERhNzKIuhJEMVMQOPYdDd+Bpx4nILi7rPkCtnJKQwCkE6MrCBHbO6OystpK7JGMpNRitXsWOztmJiEu2SASrgqTpqRHgDk8NKDKrKnNPmdbD4WGIoTit4u6f3wdjldrbEazJElQYM71PJvxp6NXMctxcXZlU5EVtGQ2BbQ+HxrcWRjWaiGGHsYN7rLbt+u7Kq8OsSI1FZndrQxKSjFyeyCWsS9tuivhrbodD9a2ZmRB1WdYB7VINFp1v2VNHwf17vvYVcIyXWUndP79f+GPYpRcBfRbkSXXVHXm45feA0+sFOpklKD0Ong+krNRquz2UvlJcV7+V+F96N+nz2V+j4tc9qIBIz5R/jT2jtoE5PNnjowuPws5xz0lry4PvTLxthYO+Q9tujDaiDKN223G7uNdPD9K1JRcJLN98jyTr5Z2qdiXft4imM/JDn/pLN8K29SFEHvAIAPapA7ONc+tKjKV0nF+46tKpUcbq0o+Jzu0NobQ2cwS8wuLuBzN8YrSrSgtbNCH4XCYtvLHLJb3SFdobXfanQ4W2CLhuFhmAiUtudComh1qkKiSirMNhcF+Ccqlrq3C7e/Irf8AZfaH6Jv3krHVVvuwb/UMF/L3S+hR4Ky2cHKYG8xu4a0KElc72EX50S4QUdnooIKtDbGIoOorLYzGNwypWJSsMRpkglZUgvVmZa1mBypBM2hHYfdVrcVr0rQfgyC4kKqDmb/mVtgeyhzf5kvvmeKqfpQ8Zf8AqTs4YXejytGWBrzjIZ5fzpLrOrqO6O5+FWLwlPJK2VL12d/Pj9Sq2rZe2YYEe49x401CcZq6OHiMNVoSy1Fb4Pwf2y19G8IzosaROu7QEiaSrPttHpOjY/kRmzoNm444O8LyQcwK3be5biH1weU8+Bg86Nh6jkrPgczpfCU6UlUhpm3XzXzH8D6QC3iL15SXEA2FZjGbQqWXhr1yOaxrM0ycYSu2z9HxGKZs91kuEsdTJkMe869w0pOrUcqihwujtYOhGnh5Yjd5ZW7rJ+/QqvQ7DXelFzcp3lvrjUmOJ3jX31rEThbK9zPRuGrp9atI9/Hw+pcbZsK2ZyQCAZncw+yTz5fMDoVWnlHeksFCdPrVo1719eXoeabZwwR9PVOo9xrqwk2eca4hMNhGFnpGKKpIyywlomYEyPeeFMwoSy9Z9sA6yz5CNhwdxmsqaZpou/R+4yYiwyRmF60VndOdd9EyqWjAYibhSlNbpN+iPQvSPZdjGAm8htXOFwCRPfvjs1HdRZUezl3XvPM0OkJRqOpB2vuv2v5pnnO0tlYjBmT/AEloHR0Jy98jW23b791LSUoaPY7dDE0cUtNJcn96oVtqH1Gg4gwBPORop7dJ5Csd6H6OMq4dZVquRe+iwxOHuRbIKtq1m4JV+3LxO7rIZ7a3SpRnK8tHzLlX6PxWmIVu/f79zPQbe3EiGt3rLcQpzr7cpHdrXSWFm9bxkvR/NHLxHQdGzlg62nK/2/eUG3PR5sZqovXDwGQAeLf60WSoKOSoorvuKYTD4jD8F5XZyuw9j4jBbSw/qhszZSCGWejeVJGkxw7a5M6EVUVneL4nSr4u2HnJO0o+fFHq/wCesT+jt/P7VH/DU/5M87/q0+cfT+zwjDbQBzJB67yD4zr5VyqdPtRfI+g4Z/mxHLYptnoqa0DotCY3CIzbSs3HacBgLS0562HYwJi3WOssbyoiy1tTMuANhR4yFK0ew/BiG0F6kjgZ89D7QKlaOWpfn9/U+fXvTlHk0/VWf/qT2Xiyt1OTsk9hzDWla1PMr8hvo3FOlUUOEml53Vn9f6Lrb1klG0kAMezQE0pSdpI9FjoZqMr7JN+iKTC+kK2bZtorCdWZtSTxCgbhPbTdWlmaZ53A4+VCDg9uHc+JVXtqXXaQdOAmiQgoqyFMTiJ155peRobVdd/sNaFy82P6SEIUaWRwyssFoDdWQOzfS9Sled/edbCYtU6Lha++n3wOn/OIsojRJKmADxgbzS8KTnJo7GLxio0FNrWVrL36nOY3GvcbMxnXQDcJ5D476ehTjBaHmsRiqtd3m/Lgvv1Oa2xezPpuUR47z7aapqyFpGGw8HQsFGpAJCg8zw1IHlTTUrO/D3AbpStcnbtSVYBpkDQTM8DQpxatI2mm7D5xxt9GOHSo5ECZQg7zrVzSumDnHNTlHmmj0bZXpDbuCFua8jofI6HwoixVKPtaHisVgqlJ3lHzRPH2TcVlyIZGpllP90R50dV8LNe2Xh6sack9dPP4nnmO2FiLDEqkpyBzactwNVXp0ILNRmmuKbR6SjjaNdWb1CbK2otvqlnTnbYgD926Cvlr20ClUpy1Tt56Er4Z1NbJ9/H1R1uC9KYjrP8AsG8g/u3I8gKbUL8n5HPdGtT9hteafxQfHemByxLt/vGuZfHpHK+yiwjSjrJpeCXx0J1eJqaSm/X6I43aG3i2ItXGbNkeYUSAIIMHcTrwmg4zE0ZxjCHB3ffpzHqOCcaM4pbridB/tfZ+037lJddD+JzP9Mrd3qjhLbJmGVRqRB5c6zltJWPb4X9aPiWSVbPTUxm0tBloPU4nRYP0WxjrmXD3I7Rl/iilZ14W018Ewn47C03aVRX++Qve2ddtNluW2Q8mBE9076T61PU6NKtTqRvTkmu4YWyKXdXUy5CuItRrTFGpcJF3FXFPQeoOsuyxO4sgjw8+PgYroYuneiprgz5dCaji3CWzSXy/vyEcHvHNXU92oPvFc6XsvwDUE41Yp8JL3M7nbRixd/UYeYj41z6K7cT1ePdsNU8H79DgLuHE10zxoI4IVCE0wQHCoQb2ZhxnUcy4/iodX2WOYBXrxjzv8L/I6PbSxbtDsb3Cl8P7TOr0yrUoLv8AkU6WkeQ94WdIVjbe5J3GAg5cTXRpUpT2PP68AJ9H8Jxx58MJd+LCmlh6l+BnLJ8PeK43bTi0LCqihJUsi5OkUiJuAaFoG/fEcqJPFSgnGKt97Cf4ePW55O/yK/ZVu8962mGzNeLZly6Nn36HhAB176TfaWXfmMpqN2BxBYscwIZSQQdIIMEHtmtXbZrQefEs6Wlsi+HAYXmNxijHMcpQCMoCwDJ/nIRm2+RlqNg+1LWW0WBbN1ZOdjxAO80arTio3SBxSvsUX0h/tN5mlbILljyINcJ3mpsXZEJqFk1rcUrFMsdn4Nbg1uFTOuhIAmJJG4a0aFOMk2uHIxKVnYf/ADAP06eZ/ChdZT5S/wASrT/hL0KrCaOvfWaftI6WG/Vj4l9bFHaPT09z1v8AJp6NItpcVcUNceTbnXIswCB9o755eNcqrPPNx4I5nSeMnfqYaJb956AK0jhC20MBbvIUuKGU8+HaDwPbWKlKM1qGoYipQmp03ZnmO19lmxda2TMaqeancfh3g1ypxcZNM9zhMWsRRVRefiVGJQdlFpJ3HYtlViRqa6tJaILUXYYg4393uruOObDSX3ofIcY7YteSFnSGn7S5vEGD/eVvOuEtmjqVH+ZGpzs/PZ+9NnUek1w/RrgBgnKB+8D7gaTw6/MR6PpV5cNLvsvejkcQwBHaN/wroHkzBUITLAVCE8C0NaO6LokdmcjXwNYqK8WHwk8leEu9fQ6P0hf+zH63+GlcLuztdNfpw8X8Dn3ujkT4eNeiw6tTVjzMsRCLsYLv3fM5aM7oH+MS2idIvors1lQjaKiVGYHDBzm1nXNA5UnUp1pPsKK8bP5iP4hL2pP/ABkS2Ns6xhL5u2r3TkEFGNnochBmQUxAJBHVKkQQTu4inQqxtmf+KT/oJ+Njk7Mc3jdfJsDtPZdm+5uXGUuZJItBZJ3kxd30ZOkv2S9H9RX8ViOCS8//AJFBsHDjc0fsD/OrSnS/g/R/Ur8XiOK9/wD8kcTse2wg3RB4FU/z/mBW3UpvRxl6P6mo4mrvb3v/AGiTejNrhcTyt/59DfU8pf4/2bWMq/x97/2A39Gbf27f/THH/iNay40bfu/xfyYRYuo+Hx/2kbXopYf1sUtkiJHRXrgJ4wQDu79eFChQrVdYQsu92+IeGKivbYltj0dW2wWxf6dcslzaNqGkgqFZiSIAM6b92lFjhK6XaSXmbeKp30+Axst7lrS30dk9GVZm6Rwx0klYaCewAad1U6NWnTnHLmzcmk0vHQXrOnUalK7s7pbfQX/NLf8AurPliP8AJpfJX/hL1j/uH/8AVqn8X7vqVGE9de+rp+0h7Dv82PidBbNM2PS05Hu/odi1fB2Cp3W1U/rIMrDzFecr5oVZLvOPjIPrpX46l8t2tRrNCLgSF2jKsYyHn/p7il+kgTqLag95LEDy99Lyhnk5Hreg6clh23xbscljLoo9Gid2CKu61dCCsXUejEzvrtUdaL8z5F0j/wDov4fEiqZk/VZx4XLZI8jab96vPfu8V8P+TpPWjf8Ai/c1f4p+pc+kd3+hQcyD4BT+IpXDLts7vTE/yIrm/kznH4dwp084QFuN2nt8qhCSgD8ahDD6vidfOoU78C29IMVm6JucnzCmlMOrNo9B0zNSp02uOvuOW2goS8cw6rQR3ERI8Zp9K8dDzzVmEtIjdVQGM6EZpgTuHI6HUToN2skVO+iRa10GWw0AdQKRvMmT3gmB4RupiOFbWuhrqr8AHQg8azUoKDtf3f2YlHK7DGD2T0lxEDAF3VZjdmIE9u+gVstKnKo+Cb9PMqHako8xbGYIW792wSJtO6FtwORisgcJiqw7jWpxmtLpP1JNZW0RGDX7S+dH6hczGZcjLuCygGd9aWGvxMuolwFXYDnQ5Usu7CKzV7EenX73srGRF6GfSF+97KmVImgw4QW1udKpLMwNsZ+kWI6zSoTKZ0hj3aGsq17WLsgHTr972VvIVoGQazFb6mrukdWHVxd7D+Fck1qCnm7ex06E3LY7j0R9IWw7KiKzq/rossc32kEetG/WNOFKYrCxqtu/g3ZD9bD06tNX39yPRcNt4MAeivCTEFAD4jNoO01zpYTK2sy07zkzwTTtmXr/AEK7X9KWtIxTD3SR9Z0yoO0kHUd3nW1hdryXrqGw3Rcak0pzVu56nmWMxxd2e44LMSWJI305GlFKyR6uE6NCCgmkl3ipxSzGbU9+tEUO4w8bRvlUtSNxq2kYqz0F1aTXXor8r1PlmP1rALWMyBhAOYAdxDAz5Zh+1XnrXaY7GpljKPO3uf8AyL3sRduATmYKIAjQbhy99SMFHY1WxFSrbO7227g2zsYhOW4qqeDQAD36ad+6tASzv4BTwynmNPMcahCnbQkciR4gwahDTP1fH8aosJjr027PYCPKB8KDBWnI6WKnnwtH09NBXbFrPZS4N6HK36p9U+B/jpmm7Oxz2rwvy+D/AL+JW7JaLyHtPuNNU/aRmn7SLrG4kASTA+d3On5VI01eTGZSSVykfHmeoI7TBPluFcytXc5XWgtJ3dyAxF4EMHcEGQQxBBG4iDpQG21ZlF1s/biuSuJVSxP9oVGpO/pNJnt8+dVHsqy0I9Qu1dkpkNy1AgSQDKkb9OVGhVezKaKbCXidDwp7Dyu2heqtB7ZD4cXj9Jtvdt5LgCo2Q9IVGRieQPyd1BxUKktIO2oSOkEVj4YjiDWnRtDPdeHEvNwN7OwXS3VtG5btZjGe62VF0JliAY3R40rOWVXsbSuAt2idwJ7q2k3sVexLoH+yfKryS5EugyNMAaeVFg1OWVSfml9WHhKV7IYRLg3N7TR/w8uY3HrltL3lhs/bF+w023IYwN2aZO4UtWoOXZevqF/F14aTd133+pbYv0k2gzFTeKQSNGZTppqFO+rXR8YvW3xD0q1eprGMUu+/zb+AjduYi5/aYhz885osaCj/AEkhlUK8vaqJeEUvfoCGz1+s7t3tVul4hF0fT/fOT8x3GbLtWXsqgi4qG5eMkwbn9lb13EL1j+vStBupKVvZWi+YOjh6UcUnTVlHfxe3zNu9NdWdaVW6FLl3KdN/urNXFZKfVx3+B4KtTU6mZkxYVBmuHuXiY+Rrw051zTQT6YRGYqg4KSq6ftEE9+ndUIQ2rh1ZCxIBjRhrI8DrUIUVpbw6q3oUcRcIEdg3+EVCDiPwGsceHiahCUSOevCfwqFpN7Grz9RREQzCO8KfjQ7dtvuGZy/IjF8G/k/mMbKuAlrb+rcUqfge/fHbFbfcBpySeuz0f33blKyGy/W3oxEcyNPLto8atrSRlxcJWe6A3GZzmY/yHIcqHObk7spu49szZN+/pYtFhxbQKO9jpPZvrJRvGbMa02Vrtpm1lUcuRAnXqx7avK7XJcCbSn1gdRoRvB58j3dtUQbQfR7TCEdrqsonXKpEFwODcp7+FajDMU2I4ManuroYVdpgKuxHEOQdPnQVKzabaNw9lAWuE7zNKuTe5uyNho3gH541l3exocsbQVBAtiSZJJ9wjSroylC99TEo3C/ngfol86N1xnJ3iVkdYd9VQ/Uj4jEH2kPs4Ak116klCN2OOeVXNYNnzC4GKONUI3qeBFAjSlKGdu0nt3IHCDqtuXkOW7mYTuI0YcjzHYaFSk/Ylujqwq9Ys2zW65Pmu5/0FW5R7Bo1Cx2VllrtwTbtLncfajREHazEDxNK4ubhC0d3ovvuCOsoQc3wEzeZiz3DLuxdz95t8dg3Duo1GiqcFFGKF4Q13er8TQM0Rqy1NupZXDJYW3muudN48pPjvriVLOTseVe5UYvHEsW+uf7g4KvbzPAk8d2CA7ByXsrQ2Zd/3jrM94jxqlqjVSLi3EtsSnSW1VVGaVzTuCqGAI7daswD2Tse5dci0mcgSdQIEhZJYgASw41CMtW9HL4GY20ClcwY3bIQqAzEq5fK3VVm0J0E7qhRZ7G2diMM7XHtgWgVt3CHttlZ8jW5CsTrmTXk9BxEM0NOB0uiq/V4hJ7S08+H08zPSxQQt0ASOq3cfVJ7jp40DC1N4s6PTeE7KrLho/Dh79PM4vENDhhpx8fmKdPOo36QoGa0wGrAjTiwygCOeXJ51lPdchiqrxjPmrPxWnwsWmwPRgMOmxPVtASFJjOB9ZiNycuJ7BE6Su7IAWJ2x9Kb6NaXorUQCvVJUcABoq9lXib4ez3KqdkDtf0bs4dD1wWCncZ4UChi3V7LVikc3gUm6yHVQJA7erJoxoYxOBLNMjUTv3DT8aNGolEywFzBlNZHL58qbwk1Kb8ANXYRunrc/kVqvuzdP2UCJncKU3CEWQ1VmQl0ZHAVdmQjnHKpcg6li1E52kbhFVSnKNWLa0CaIxRmMncN1dejF1pdZNaLZBEnN3ewylOWGouxlwEHMu8bx9ocQaUr0W+1HdG7uLzx3+K5BbV0MJG73dhq6UlONw8KkZK6CrjWZehEZA4djxZwIQE8QJJjmaBGkqlfrP46FdZ1klDgtX3vgiZNOZRlyGdnuM2vHceRpLG05OGgljFKVPQFt8vA0MDjG+OPidf2VrjnJObYyahGGxzxeB5EDyNZj7KCVvbZ0Gz8SuYgQdPiOO6tA7aEcNi2tHMjsjDSVYqeW8VCg1zalxiWa9cYkZSWdiSsOsGTui5cEffbmahVhc3wSSW1KhSZMlVy5VPYMq6fdHKrKsXQxwuWiGM9Ug944+cGkOryVNOZ6xYyOIwLU3q4tPxXH4MoMdhmOXIjnfMK3Z2U8eWRZ4K2oUNetsCrDJ1GJBZYJgDdCj2VlJ5vIPddTbjm+KX0B7XxhIKgMV4zJM8NKcpdXT7Unr3GYpR1ZVYbG9GSQrAkRO74UviJKrK9jEsreq9/9Eypuzku9Y/UaBPYG3HxipCcYtXXmb6pT0pvXk9H5cH7n3C+y5+kOCCCAwMgg6FRqDqN1U3d3QJprRjN0vnMZTpp3aUWMI5bsy3YFfxDFFQqgyljmC9cluDNxAjQcNacwlNKo5J8PIBUK8jrfPZRKy3Nw9kGEgmlErMJc1d4VUiImWq+BLgoodmS6CRx4V0YUYzqZktL/bNt6XY4tdnJYPF6ExWbBUyYNVlCKRC4AssDE6FeZ4EdtK1qOV5qe70tz7wc5dXeS2e/iGtWSnVO/eeO/keIo9Oh1ccvr4haDtHxCE1vIMZjab6FOGhnMGuE5WM8B7xXOxOmH9PicaatUa7you2+so5kDzNcZ6I3BXkl3krNoMzOeLNHcSdakdi6jzSb72O4TSTVmBFsUVeQeJ+O8HfVNXNRk4u6Oj2LhcNfEFSlzgBBVv1AwMH7s93KgVJVIarVHRwlHDYmWWTcJd2z8L7eHy2Z/MDk/wBHctkcJlPDQGsLFR4oaqdBVY6wkmu/T6it+29pijRmB149uhpmLUldHGq05U5uEt0BfFtzrQMgcS32jUIDa4TvJqEI1CGis9vfrUINYYhiA0Zoyo53ryVjxSdNfV3jSQcNZdV6DEZqr2Kj14P5Pu7914HP3ic7hgVIZgQd4MmQa7FOzinwEJxcXbiRFymaFnJpGXFgnbWfnhWcTDKrm4rgQNw0jdGspo3DWWy7Excq9CrG8/ZVaEsG2faa44QbzMDuBOnlXVwanKbi33+BrOuOxa4XZRYb4I3giu06E7K8kFjOnHmEbZhHE+X86E8LV7vvyGYuD4m12W53EeRFDdCsuHvNvKuKN7NRz0oRUf6hLIGjtRiOq0jeOVajCSgqjXavok+C39foKNqpVyt9le9i+Iwty0RnBynQHfB5VU605SzTQaK6p2TvF+4OMHc4IT3a+6sKtHiho2uDucUYfsn8KzKrCxTlYcwmELdWDug6RxpCtRlVpOMNzkVaijUYvi9mi20uYiRA3liNAPMHsrz8003F7jVK0Xnlt8fAFawhbcPLh3VYJu7uRxOFZIAMagnu+sPKoUU3QljIE86hCww9t0II8qhE7ao6nZ21M5DjUgxcHHXc5HCdx7YP1qRrUUtj0/RmPlUWWfn8n9eT8UVe38WGv3O8fwrTVH9NHE6QVsVUXf8AJFYbtEEzXSVCGukqEN9JUISFyoQ2LtQgHbKF7udYMqk6gS2UBideJ1rsYXC1XRTs7cPAHWqxc7+HrZXETYYbxHl8K6WBw0lN3XAE6iewK6tTpClaKXeagyAQncCa5PVS5G8yNG2eR8jVOlLkTMjAKz1bLuZVZCXO7w+OwFlg6YNAw3FsVdc6iNyKOfKvRw6PqKWlTXuivmwTceb9Ad/0tTpQ6YNYkBlFxyGad+Y6idx8O2ZWp16UbLNK73slb7ZGk9nqWA9L8MfX2ZdXtS8W/it0vbGR1bf+P0ZNeDB7T9KMF0DizYxNu8VhM/R5ATAJJGugkjTfFUq2IckptW8GmXqhr0Z2jsq1h7aPiHW5ANz+hYjOd4BAMgaCeyhTxVXM1FK3DUijPgWtzE7JvKUONSCIIe3dTyJQAGo8RWtrD3r6l3mvt/QodiCzbxRwbYmzctnWzfDDJrJyOfqkxGu494o1PEVMmkXpw4hJVHbQ6656OqR1b9jvF9PxqljrPtQl/iylUkufuB4fY1u11r2Kw47Tetk+/wDGo8Vn0pU5ejMuT5fAFtM4A6rZGJeI6Q57VsDtuGGffuRSO0Uq+jpV5OVRKN/OXotPVmE5Xu2cxicXbQELDGdIBVV7FEkx+sSa6NPoCi12r+pHV5MrcReNwQQCBviQQOwzXL6X6NpYbJ1V7u/ebp1HK9yswjoEYpE8YkmRP2ju/GuEFNW8eeyoQiu0gGzFSrA71JBYcojUESNTVSSaswlKo6c1NcBXFY3M5cg9bXhyj4VUI5YpGq9V1qkqj4kGxY4K3iyj4VoCCOLPJf3gahDRxR+55k+41CGhi25r5E1CExirh3HyT+VQhd+jtq4bqtcVMm8m6gCnUcCJPcInmKYwlB16qpr7XEqUkldnWvjrO4Wtln/8zD3XK9ZDAyikouol/wCS+gs6kRW7ibB34TZzfq/SLf8ADdoywtRbVKi9H8iushy95K1gsIwn6BYP6uNvr/FNBqUa1/1ZecF8i1KL2+JjbMwvDZgP6uPP+JKwqVZf9X1ga0NHY2EbfgcWn+7xlhv47dXlrL/qQfjB/ImVMifRzBH/ANLaQ/8Aswr/AAFDdOs/3U/R/QmVciP+zWC+xtLywv8A51XVVucPf/tJY4BIHCe+lIVadLaF3zeowoX4hS5PHSpWxdero27dwWNOKCK7faPmakcVXjtN+oXq4vdGLiGZgSxOX1Z1j5PurUMTVqSU5O9thfJBzfJDn56ufaDd6qfeKaeLk97en9mZdV+1Art97mmRB2i2ik+MTWZ17/tXoDs+Axs6xkuK7Q0Hcdfn+VHw9W7UX6mct3qzoH2lZ/Q2/FR+FdFUqn8n6hLS5kBthF9VEU/dUD21rqG95NgmxHF7VuXNJIosaMKaAznlFbNkzqTHLnVSqpK/AXlV5Bhiwpi2Mx4jcv7RO+vP47H0MSurpQztX14Lvv8AaCU6dSLzTlZfEq1t5jJZnYnRU6qjjqdwEnlpFeeoQhNWd3LhFfFsdnJrklzYddlvEyoP2dTA5ZudO/6PiHHNonyv89hf8bTTtr4gL9p19ddOe8eY0rnVqFWi7VItfD12GYVIT9l3BWimYSoI7RQjZYi7a/RW/wBxfwqEJjFoNyIP2VHwqEN/nHkAPAVCA22iedQgC5jjzqrogs10kEzw+Irr9CSccUpLgmDqeyCFyvZrFMXymxdNaWK5lZUSXEkcTV/io8SurQRcc4+sfOtKvB8CurQRdpXB9c+dTPTfAmQIu2Lo3OfOqbo8Ui8r5kvz5f8A0h86H+T/ABRLPmykArw6qvmdHq0bC1tVSdUwi224E1vrHzNdVINbwpO+tQdo2YNUXcds4UCiKbCqlYYAFETMuBKj0pWkBkrGLaNdiNZtasxOWhjWqJGrbYRnUtojYgVJTvuAbb3OmwOCWxhGxDgG44i0CJCzuMcTvbwivOY6vPF11hab04/PyXxHKUI0odZLyK19hxh87GC56oJ3zrLHjpJ/1oFa2f8AB4XRfufPxfJf0ajK0euqeSFsPhgghdeZ5/y3+ddnBYKGFTy6t7v74HNr4iVXV6DK2edNOQs58gpAXf5cf5UOXa0epSzN3RzWMsr0uggZ2EdkSBXi66y1ZLvfxPS0vYj4Ik2DuZEdUlSikwJ1jrHdzmunhMLTlSUpK9xapiYqo4XtYSe8RvAH7K/hR/wlL+JtTb4kOnPMeQ/CiLC0v4o1mZhutz8tPdR4UKa/avQl2a6RuZ8zTHVx/ivQq5FnJ3knvoi02RRqt3IYTVORDJqnKxDU1lTZLG5rXWsljCaqVR21JYjmpbrnzNWIKK88kOpDFq2TREHjF8Bq3aA31tBlAYD1pM11ZJQTREYcbB0s0aICSGUtUaItOLIuYp6DdhWcQDKTTEWIVHleoW1ha05gJVBtRpGp5b/YKHoncFKTejJ4y9cyjMSdQBPDj8Irk9ITjh4XopKTdrre27HMJetK09UhXaW2MQiKFvXLc8Lbtb/hIrz8qk5u8m34s6qjFbIQsbRxG83Lh7WZm/impGpOHstrzJKEZbotcLjkOjMub3nlpTlPpLEw/dfx+7i88HRlwt4FDisSDczffYmO0RpSU5ucnJ8XcYjFRiorgXWzceq2EzMBEKBrrA1+e2mIYyrCChHSwvLB0p1HOWrYpisdcJ6jGPu/iNaFKvUl7UmGhShD2UgWB2viA4BvXSJ1VrjkeKkxQ02tmEGr9gFjmUE68Na6fR2Jn1qhJ3T5i2Jj2G47i74FeC16OyQgq0rbkH2enL21RaryAnArwmpcIqz4mvzaOZrLZf4juNnZP3j5Vkr8T3Armzo+t7KtG44i/AB9FPMVAnWI0cK3ZWJak62JH6K1CyLkTrYm1CiuBc60UEF7lWswxCS4BUk1aYxFNhFFERvKMWzRkyuqb3G7VGiClSGM4o8EAlRMydlOwWgjWppI2VPIUZHExMbajWCwT3WCIjOx3KoLHyFYqTjTWaTsu8USlJ5Yq50Dej9rDgnG4qzh2gkWp6W6e9EMj21ya3S1NO0Ff3DlPo+b1m7e84Pa21rRuHJaZyREuSBAiIRdSNBvIrh1akqs3OW7OrCChFRQi9+4eSD7oC+7X20M2J3b/OSe01CGWL2u6oQsVUFVMfWMeI19oFQgleuQIj/WoQAMR2VCDlm7c3qx7iZ9h0qECrtHKYuWQZjrLNs/FT5CoQ7HY2FwmJt9XGW7F3QLbxAKA6fpR1QZ0iuxhulckVCor2431+/MQrYLNJyi/IDtv0fxGG/tbTBT6twQ9tu0OunhvrrUcVSrew9eXEVlRnT1kVVuzRmDlKwe3ZjXcKwwea4O4w4VLGkhG81ZbGIrQFkqJm2zZWsuRRqRWcxdimSvPXO3FXGbRq7jdOyGENTMNRsxi2taUhmERi0tHjNB40hpLRNNQdzbopLUcw+DpiAjWWtkP28HTkWcmskiNywq9YiQASRMTHCeE1jF13QoOa34eJyZ0nUlZrTiU20vTrEMDasRhbJ0KWJQt/vLx/pHPiB2V5SrVnVeabuxiFOMFaKsU2Etu8lVJkySBOvGTzqU6VSp7EW/Ak6kIe00hpLEGGOWTHb3xypiGBqOVpWXx9DMqySulcsBsdT9YnugfjXTh0RTXtSb931OZPpKd7KKRpdg2Z1UnvZh8aOujcOuHvYL8fXls/cDu7Isj1VjtzMfYTWZdG0Hoo282EjjK3F+5FjgfRDE4lc2GCMiNBzPBz5EYiI3dYedcCvTVOrKC4M61KTnBSfEQbZdmAWBOgkZo1jUads118LgaEqUZz1b7zn1cTW61whw7hK7s+3PVsn99vxqquEobQj72M05VFrNj+D2ECJIZPEH3ipT6KjJatoWr9IqGkNTd/YrAdVge8R7podToia9iSfjp9SU+k4y9qLRWYnCXFHqmOzUeykquCr0/ai/LX4DkMTSntIlsj0oxWE0s3WRT61vR7bDiGtPKme6aVT5B7F9b2kuJXpFs27LDRxaLBGJ1zKjT0fcDHdXc6NxU6jdObvpocvG0IwSnFArvZXWEVYSvchWJMPBcWAyxrWAzZJbR3mo2UQZJ3UNstIXzDmPnxoeYLYqVFcQ66Ywi1VxiAxbqXHqTGLdVccgNWWosBmM0WmEE/zpyEip1Fx1ZbYdRxpumxOorjZIGnGn4O5za9LQ53b+JzQqEgrOc7gCdMo4nSvPdJYmVWq4cI6HOb4FPsDCqbrZlDQsietrI11q+iqcKle01fR7+Rz+kJyhRvF21OnLADkK9Rbkees2ylxCS3VGlBqQTep06VRxW4yiPwNEbiAbT3DW7VzsPfQ5TjwNwp32AXDEzGnCR7edCUtczYSVGWyPT/yTX1WzjgfqZbp/atss/wDRrydV3nJ97O1FWikeS3bJGQQT1F893wro4NSlBckCqNJ7DGHxJT/0274rrQWVCdSCqPtXMbazz6hjy+FGhUtuLyw1N7KwZNo5juIrSkmCnQy7DCjN3UXMgOWwlt3DIbLMVGYAQY1BJHGuT0rGHU5rK91rxHsBKXWWvpbYrdkEpGsppnUbyPH3VwqVWdKWaDszqzpxmssi4uxPVMgnQ8xXp6VfrKanzORKhlm1yE7vLzq3M3GAJUk1hzCKAwVAHz41hzLyC14iI51hyNKAHKPn/WsXN2KNWrjHTiwiNUuHgw6GqG6bSGEarQyqg3YHOiR0N9Y2WNm7HGKNCdjaYyuLPzvpmEzE6ltA9jFtypynVSOfWvLcovSS4S4yAAkdbh1uZ7Yjyrl42ipVbw47+Jz5ws13mtiXctthBzFiSfARHZXS6LyU6Tvu3qczF0pVJWDXMWeVdTrYiP4d3sZZxJnhS1SvFBFhZPQd6YgSxAFCVdNbBo4NR3F72LZtASB36nvrDqjMacVsBZOVL1Jtu4XIJY3aF4XHCXblsFFRgjsmdQNcwUjMJY764lVWm0FHsPiBcVSSCQqyORj8aaozWRRTIkib3WOiifh7adVWrbRAXTp31ZEMw4COPzNX1lbkZ6uiGV3bj4fjWb1b7kcaXImtpyfW07Kj6x7yLSpraIdtnuwgtpxHOqcHLRyLzKOyKq1sK6jxnXo5365o7oifGkngpJ76Go1E9ixx2LQCFVRpA0Gg5/hXUhKKjZbC0qbvqV3SCI86tyLUSduBrWc5eUhdu76zmLURQ3J1rLkasRzHnVXLsilBrlDaCKageLGEqBoyGEapewxC7Dpdq8wxGyDI/wDrW4skpNjFu5FFUwTZM4rhRozFajFMVcndqfdVuSuJ1tUQsAjefbRYSsIS3DlwdKJ1hAF1sp0MnlU6xcSmpcCBxlw8J5VtVktgfVX3Zr6c32ffWJTuGisuwRccx3r76XqVUHUmxbG3FLKzcB3aya59bWVyyeFxagwNx3j40ON7qxCQxxAgU/Gq0ZlBMMl+dPOmVVTAunYds3oA5/hVSqJFqIymLihOqEUCbYqd1RTuRpi2I2gQDrurSmynBFRcvliWO81TmRIjbcnjVdYy8qCtiTVdYyZECF6rzlZSSXAeAqZirE+kXkKvMSxRBa5wwmEWoETCK1VcNEOjVQzGQZDWgqYdWq0zWiJdJRYgZy5EC01vMLyNho3VeYXkrmZprSmwLggdzE8F860mCaBKvGrzGbBlnhUzF2DZoqZi7Abt0zS89wiF7y5hBBrNk1ZkBW7QXdM9tXGKiQMhjdV3IOYdCPPX58alyBVaNfx+YqXITLjdFXdE1BtcI3VFIjE7xJPGPn+VFuYBnWstlhAahZFxNUyXBMSKoskpqXIbzVMxWUrTS5tElqGkSrLDRDLVDCDpWg0Q4q0ElsY1EF5bErdWBka/lWgTNXfVqIDMXSigRhahkMd3zzqFoE/z5ViWxtEKGWQub6hCJ4d9WUPL+Pwqiya7/AVCzE+fOoQG3xP8Jq47lMFe+FEZQOoUiQqiArlUyzE3eVUWAuVTISt1ZDdWQ//Z</t>
-  </si>
-  <si>
     <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/2wCEAAkGBxITEhUSEhIVFRUVFRUVGBUVGRUVFxcYFRUWFxUVFRUYHSggGBolHRUVITEhJSkrLi4uFx8zODMtNygtLisBCgoKDg0OGxAQGy0lHx8tLSstLS0rLSsrKy0rLS0vLS0tLS0tLS0tLS0tNi0rLS0rLS0tLS0tLS0tLS0tLSstLf/AABEIANcA6wMBIgACEQEDEQH/xAAcAAABBQEBAQAAAAAAAAAAAAAAAwQFBgcCAQj/xABPEAABAwICBAgHDAcIAgMBAAABAAIDBBEhMQUSQVEGBxMiYXGBkTJSkqGxwdEIFCMzQnJzsrPS4fAXU1RigpPTJDREY3SiwvFDozWDwxX/xAAaAQACAwEBAAAAAAAAAAAAAAAAAQIDBAUG/8QALREAAgIBAwMCBAYDAAAAAAAAAAECAxEEITESE1EFQTJhgZEUIiNScaE0QtH/2gAMAwEAAhEDEQA/ANxQhUbjK4cSaNMOpCyQSiQnXc5ttQsAtYfvnuQBeULGabjmqHjWFHERiPjXDLralWcc0t7GgZ2TH+mrXRYl1OLwT7c/BsKFmUPGfUFof/8AzHFpF7tmB7hqXUeOPOC9jSPFsD8ILg7iC0KtRb4IGuoWTN486XbTSdj40q3jxov2ebyofvp9EvAGqIWYN47qD9TP/wCj+olG8dVB+qnHZD/UR0S8AaWhZwOOfR3iz+TF/UXo45tG7p/Jj/qJdL8AaMhZ4OOPRv8An+Qz769/TFo3/O8hv30YYGhIWe/pi0b/AJ3kN+8j9MWjf87yG/fRhgaEhZ2eOTRv+f5DPvrz9MujfFn8mP8AqIwwNFQs6fxx6PH/AI6jyYx/+iSdx0UOyGoPZF/UT6JeAyaUhZkeOii2U9SeyH+ovP0zUxypKk/yvvJ9qfh/YXUjTkLMBxwRnKhnP8TAu2caj3eDo6U//Y0f8U+zZ+1/Yj3Ir3NMQsxquM6pY3Xdo3VbvdO0ebVUe7jin2UDO2c/00u1PwyUZKXw7mvIWQDjaqzlQxdsrj/xV84BcIn11Ly8kbY3co9mq0kjmEY3PWlKLjyicoSjyixoQhRIgsZ90L/hfmVHphWzLGfdC50vzKj0wpx+JDXJmGjH2iHb6SnejxrG6iKWT4IdvpKlNDSL0ep/x4JeDp0Ty0jRKOb4FltwUDwh4Pw1N3Easn6xuf8AEPlenpTnR1V8A4bWX9oRwYc58XKucTrudYbgHEeorh01znPEOTJDTytm4IzbSegZob3brtHy2YjtGbe1Rdlt1RQRvzGO8YHvCgNJcEon3IOPSAT5QsV0VXeuY5/gVmhsgzMEK5VPAhw8Fw7z6wo6XgrKNo83tUsS/a/sUOixexXkKXfoCQbR5vakXaJcMyPz2pqE3xF/ZkO3LwRyE+NDbM/nuXPINCl2rP2sXS0M7LtkROQ9XpTxrQMglAl2p++wuBuylHyj2D2p1G4N8ABvTt7yuV6rI0R99xZDErtgXLU5hZdaYQISeDuBqkYGJKnhUxR0t1qjHCMtkxSip7qyUsQjYXuyaCT2C640Xo/oTrhdHqUMxHigd7gPWsuouwtjG31SSKHW6SkqZdZ2DAea3YB7U9ZGLKN0cLgC2wm46LX9KlaVtjYrkWzcI9TPXem0xcE0h3RQLTeJn/48/wCom9IVFoIMVe+Jv+4O/wBTP9YLl97uNl/qcelRX8l6QhCZyAWMe6FzpfmVHphWzrGPdDZ0vzKj0wpx5Q0Y7TP5pG4lPNGz2KjaZ+JG9KsdYr0MZddMflsX1T6ZZLzoqfnWvg4W7VK8HDqtfDtjkdb5sh12nq5xH8KpNDXWsd1lahOGllU3wCNSX5hODz8x2fQXLC/0LlP2ZsrtVd6n7S2ZZHFIvKUvcJvIV2q2pLY6dsNxGYqMqk/lKj6grZWjM0RVSFGTqUqVGVC2LgyWrYjpk1enUyauWO94ObZychdhDV6ua3uUMF6gBLxQ3TisibweQx3UpS03QldH6PJ2K0UOigBcrQsRW5jtuI2i0eTsVj0fo3oUfV6dpYMC7WcPks5x7dg7VGO4wSDzKcav7zsfMLKm28qVN1iykaLR0wAVe4wa0GIUrTd8ha5wGxjTrDquQO4rmXhc5zPgmaotcySYBvU3b1nuVXn0m3nOjPKSOJvI/ftO8rnW3Jcm3R+mNtWXvpXt5YrR04YbOIB1SbbmgYkqQpqQvLXAYW9Ka6Ko4nubDyrS6XnTSuIbzAfi262bnHCwyFytFp6BotYYbFyNbbLD35PWaZ1QjiHCGGjNHHDBT3E8P7C//VVH10rCWtsk+J/+4v8A9VUfXWLTLGTD6jNywXhCELUcwFjHuhs6Wwv8HUemFbOsl47BeooB0T+mFC5JQj1SS8mBNksbqSpqcuTfTtAYZCB4Jxb1buxTHBF4kuw+E3EdI/BaY6qVcWjVTV+r25HIoCFP8FazUfyMngSYC+QccMeg5J+7R+GSZT0XQoLVq2OGdOeji44J6nvTyCneeab8i47QM4ifGbs3t6inlQ3C4TfRU8dVH70qTZ2HJvvY3GLSHbHg5Hb6UnSyUzxBVYh3gS2s2QepwGbe0YZbdFqnXLpfAae/H6NvK4fk5lKZTBSFVFbEYg5FMpQvUVSUllF04YIqoaoyoCmKhii6li1Iw3RImdM3p9UNTGRY9Qcmxbngeuw9IFOIY1zluyl7C0LbqaoaUZuIaN5wUN76DfBFzv2JvNUOf4TiejZ3KffjBbbsr7Mp/JFsl4RwxC0Tdd2/JvftUHpDTs82DnkN8VuA/FRa9a0nJZp3SkXV6euHsehKQsuejb1Lqnpi7q3+zenzYgFgu1CjtHkucgr6xz7A4ADBuwfj0opXHV7/AElIVGY6kvTnmjt9K5+W3lkZScnlipN8F3R1kkfxcj2fMc5voKRC4TaIptcFgpuGNYzOXXA2Pa0+cAHzqx8XXGTHSsbSyU7zylQSJGOBsZpA2xabYA9KzxxXOiwRPBgfj4ftwodCXCJOyUtmz66CEISECx/j3qeTlopLX1Wzm2/nQ3WwLF/dEf4X6Oo9MKlBZkkNScXlexRtNUrKiIOabgjWa7cfzgVU9FCSOYObg9hvbPrB3hOtC6UMd2OPMd/tO8dG9Oqnww9uD24/OHQVPVUuGx1lKGpxb/suTUNFatREJG7c27WnaCkavRZ3KL4KaSHhx55PjyvbOw2EfnBX2EMlbrNy846CvOSslVI6jk0s+xn9RQkKcotKRzRmmrWhzTgHnzaxza4bHf8Aal6rRo3KFq9GdC2U6vPJnurhbH8xGaSoKiiuReopc7jGSMfvAZjpHbbNcwSslbrxuDm9GY6CNi9bp2WlNjz4/FJxHzDs6surNJyUFNVEz0UvITZuaMAd/KRbv3hh1r1Oj11lUcyWYnM/FWUy6W8oSniUbUU5Tl+kZITq1kWqMhKzFh9nmPQpiigimF43tcOg5dY2dq9BVrK5xzFmuNtd2ye/gpdRSHEnAKEqJAfBx6VKcLK8mV0LcGRuLT+84Zk9F1DsCxW6nuSwuDl6hpNpHTBbErx8l0m991zdZ5zzsjPFY3FLoG4LyKMuIAz/ADiehPMG81uJOBdtPQFDG2SeRLkw3ws9w9ZTulo3Pxdg3YMu/oTqi0ZbnPz2Dd19KfOC52o1GfyxEN9QDAJJyWkSLljENqoZHr9XtSkOQ7fSV5U5N63f8UR5Dt9JQgZ2SknHFduXBTEeE4JXRzvhYPpoPtWJBwXWj/jofpoftWo9gPrxCEKAwWL+6H/wv0dR6YVtCxf3RGdL9HUemFTr+NfyJ8GHAp5T1NxqONreC7xfwTJe3XcsqjZHpYq7JVvKJ7R+knRvBvqvFscg7de2R3OC0jg7p9smLXako8JrsGu+dsHzhh1LH45cLOy2HaOro6E9patzCMSQPBcDYjqPqK87rfT2ufudrTa1NYZ9DUdW2XmkakgzY7PrHjDpCKqhuFmWgOFpaAJAJGt62lnSLc6I9Iu3oC0zQenoKgBrZLuIwa+weeq3NkHSw9gXE/DzhLgsumo7rgpXCjRRsTZZ7MxzHXBLXA3BBIIO8EZL6C0josPacLrNeEvBdwJLQvUel6hKPTI4Gss/Nkr1FwtkA1Z2iVpwJFg63SPBf22PSuveVLM4PpZTDLsDCWHq5Mn6hULV0bmnEFRlbC4tw2Y23rqX6aHS5w2fyKa7dyU0tompLnOeBKScXsweTvc3f2EqKDbXBu02tZwIOaKTT9RHYcoXNHyX84dQJxHYQpFnCWN4tNF2ts8eS7Ed65leplB7mp7kXyLrXAJG8c4dpCS1laKHSkLfipQzoPNHc8aql3Vwc20sEMoI8JzOd1h7TbzK/wDGRxwRalnYq1PDqMHjPt3HIetTdDotseLsXnbu6Amr6cnMtdYjZY59FgpeofbHE9Sr1Or7iUY7Ik49IjIm70qA884ts0jA7O/sScixCGz0k5LSJFyAEKkYN/i/4r2PIdvpKKg4Dt9S9i+T1H6xTQmeOKTuu3+v2rghAHL17o13w0P00J7pQEOyRoxp5aLD/wA0P2wQB9eoQhRGCxb3RGdL9HUemFbSsW90PnS/R1HphU6/jX8ifBhyEIXoCoEpHIR7NhSaEmk1hjTaeUSFPUi4tcEdNiPmu9RU/o3SAvYnHM4WN97mZO6xiqjdKRzEYZjcfVuXMv8AToy3gbqda47SRs+hOFVVGBiJ48rE6xw2A+ED0Xd2Kz0nCKkqOa74J/ivy8r22WDUGmXsNw49p2btYZjoOCs9HwrY6wqIw7pPNPY4YHzLmyqtpe6LbNJRqF+nLD/o0bTPA+OUXAzyItj3Kh6Y4GSR3LRcdym9GaUjGNPVvi/ckxZ2nLzqcOlavV50Uc7T8qNwBPUDgt2n1klw/ozi3en6ml5xlfLcxrSOhSDzmkHu/wC1DzaOcMsVr+lZWPvrQSM3hzCW+a4VYlooXGwBHS3D/acPQtzVF281h+UVQvnHZmeuYRmLK68D9MxvtBOASPBLtvbvThnBd0pLYHMlcM476klugHB3YVBV2gXMdYtdE8HAOBYbjxScD5lmt9NVixXLP9Mv70ZrD2Ljwi0OAwSQawsee25cC3eNe9rbhsum0uY6/ammi+ETg0wVFw62qH2wO4OGw9OSevzXP7FlL6ZltTeMM6j/ALs3/racbev8VHyKQj/uzc/y4/nz7VHyJlg2ekXJZ6RcgYhU7O31LqHJvU76xXNTsQ0Gzep3pKYM8fn2+1eketPDQix5xv1Damrha3agQnLkVxo342L6WH7YJWYc3870no746L6WH7YIA+vUIQojBYt7ojOl+jqPTCtpWLe6HGNL9HUemFTr+NCZhyF3yTvFPcUck7xT3Fd7rj5K8HCEpyLvFPcV7yLvFPcUdcfICSEryDvFd3H2I5B/iu7ijrj5DAku45CMj7O5de93+K7uK997P8V3cUnKDWG0NZW6FYasjEXad7TbzZKTotOzMN2Px3guice0Gx86h/ez/FPcj3u/xT3LHPTUS4ePqaIaq2Jdabh/Us8I36JGg/7mapKfx8Y7T8ZD2tdh5Lh61nzIpBkHfnoSkTXgg8kHW2FuB6wqu048STJyvjZ8S/rJo8XD+L5Ej4upkfqBKjtMcIRUNLXVTXA+PF+PqUKdKRPbquoIo3ePGxh7S14PpTB8fi6vbHqfVuPOpwu6Jb4KbNPW94pfT/mwtJyZ1QZ2OsRbB988slZXnPtVLELtZt25Obl1hXGbb2/m23qUNda7HHOPoVQj07HcR/s4y777SmEifRn4Bu7oxGZyP58yYyLAWDZ6SKVekXJgIVJySjPBHUfrFI1Ry6vWUvTjmDqd6UICTa3mu7ExniGqw7SZAepupbD+Ip5G7mu/h9SjpCMP4vSpETiY4fnek9H25aLP42L7Ufj5kSOuPzvXujvjYvpYt3638Uhn12hCFEYLP+NHgdUV7qd0HJ/BCQO1yW+GWEWwPilaAhAGEDij0hvp/Ld9xdjigr/Hp/Lf9xbomOmtItp4JJ3AkRsLrDM2F7BAGON4na39bT+VJ9xdjicq/wBfT/8As+4qhp3TUlXUvqBIbON2xOdygZrWwBFt18gQAL3skafTldGLMnkaMHc2WRvgkgut03KeALwOJup21EPc/wBi7HE1UftUPkvVSg4caTZf+0THnAAawfYE5c7MqQp+NPSDSNaQkaxHPiabC2F9UYn2p4FknxxMz/tcXkO9q9HEzN+1x/y3feUZTcclYAS9kJsbC7XtLu52ClIeOd+OtBC6wuS17h2Yg44JdIZAcTEv7ZH/ACnffXX6GJP21n8o/fUhBxxRkta+kcC7INkaeu9xgn8PG1SG+tFM3VNnYMcB2hyOlhkgf0Lyftrf5R++g8TEn7a3+Ufvq5UPGPo+QgGUxXBcHTDk2WAueeTbJdM4yNGE2982ttMc1uw6iWBmL6B4N++a51CJdQtMo5Qt1geSJHg3Gdt6uv6F3/trf5R++q7wH0jFHpkzySNZE59SeUeQ1tn6+rcnK9xmtxptPUkngVUD/myxu9BQBlFdxQPjjdJ78adRpdbkiL6uNr66pda+zc7dPWvovTbwaaYggjk35G+xfOld4PaEAJxVJLQy2A22I2/juSUqTg8Lpsek5hdyIAbvSLkq9JOTAa1ZxH52lOKY8z+F3pTWszHV6ynFP4H8J+sfYgGSsIwA36voHsUVUCwHUfOVLk21eoev2KIrX5fnemRQ3dl+d660d8dF9LF9quXuw7V3o0/DRfSxfai6Bn16hCFEYIQhAAVinG7wnEsopWENbG4EP1gQ4lpu6wwNsgb3vrb1ovGBpt1JSOkawu1iIybloYH3BcXDEHYCNpC+d5Q7O7Xc0uN9l8BfCxIF8EwE3AnEsY4YG2XQwYg9eaTLAMNR7cm3bf5OJPNJv6AuixozjczG/NvkB+7tO8hcty5smIba2B5zjg1u2/SUxHglbcfCFt3OdzrZWt8oYk/nJKRB3Ns5pwccQcL3sSQcSb+c7kSa41vBI5rOaSLA25rQRniO8JKVredrR6puG4DBo/h2437AgBRhdzbtBFic8T+8bjpPlBct1SOdEdt+aHY32W2Bch7buLZHAgBoGtziegO6SB2FOJbtY1l8TZo7sSgBlGYue8iw+TgRfD1roQMOq1shu7wrOuMsT6E7ggmdqsZFrhmNmY3sMMD0pDlWc50kZucBdt8hvx6UAHJF0mryhdqWz9CcQTeENUH5NzjuJIwwOzvTGERiIkkB5xsCWm+zBKy0+oxobI67ja2BxJxN8/GKAF2S4a1jbs7811yjSLnK17kHz3Terhka0RhwIItaxFsDn2DzofyhFg0Y4XBy7CEAW7gFwlhpI6pkgk/tLAGhmrqttrAFzSRibjEblHVbNYWutU4MUdDNopsEXIVErYC4ts1zxI67ibOGsOcbX6FlEsEzCWStLHDNpwP4pYGNY4yD0WOWWxevSpBSbwjADV6ScnD2pMtTwBH1gxHV6ylYHc0DoP1nIq24jq9ZXLcLdR9JQBNucC1vUFBzuy6vWVI8pzSPm+pRTj6PWgijwnBd6PI5aL6WL7UfiknOXWjz8NF9LF9qEDPsNCEKIwQhCAKhxiaCqKqKNsGqQwuc5hOqXXFm2vhhzs7ZrHdKcHXRG0sL4T1FoJGVvku7F9IpOaFrgWuaHA5hwBB6wVbC3Cw1khKGXlHzDJRSDwXNd0O5p7wmk7P1kR67aw7wvoHSvF/Ry3LGmF2+PwfIOHdZU3SvFzVx3MRZM3cOY/yXYedWJVS+RF9a+ZlDWNIu1xvrc1t7jdcg9pSz6aQOLGlsmreRxG4Y+ENg/wCKn9I6JLHas8JY7c9pYesHb1qPdoq1zG8tvv5wTenlzHcFavcjHShzhrxnVF7/ACrkYbL4Z7E2ZZ0hLLhrRgRvOdgcP+lJyUc7GarWB1hgWnozscSmrXBupGbttbWuCDhib9Zw6lVKElyiaknwORpCSBt2uaS4jNuIOIuCMjZx2H0Js+RxFgw42GBGRzztsR72Y9xN8G5WJsTmejclaWRzm6zADa+e0A2v0bFEYhPOHOa1zSA25N232YA22Yk9gXMccT5ObYNFvBNsTfLEZD0pSKV0euXsN3HMWcNgA7r96TY+LkiX6pcbuIOBxxw37kAeRnnmxJAOricr2PpsnQCbQ0+q1u8547SNyfMFwosYaJr3QSNcxxa8OJa4YWOYI6xe4W76LFLpekD5Y28oOa+2DmPAxIOdjgR1rAqhuHb3bj3286u/FVp/katrXGzJ/g3DYH35h8q7ep5SAf8ACbi7qILvh+Gj3Dwx2bVSXtsSCCCMwcCOsL6eVb4ScC6arBLm6j9j24Ht3ppgYA9iScxWzhJwLqqQklvKR+O31hVdxCkIY1TMez1lM5Djbo9aeVj8ez1lR0rsexIY5fNYEdXqTV69keL5hJSOxQI5eUro4/DRfSxfaBIEpXRx+Gi+li+0CBn2QhCFEAQhCABCEIAEWQhACNTSskbqyMa9p+S4Bw7iqtpPi8o5LmMOhd+4bt8h3qsrehSjOUeGJxT5Mi0nxfVUdzHqzN/dOq7yXYdxKrFZROadSaMtPiyNse5y+hEhV0ccrdWRjXt3OAcO4rRHVS4kslLpXsfOE2g4nX1bsv4pw7QU1foeVgtGWuA2ZHz+1bjpLi/pn3MRdEdw57PJdj3EKqaR4F1cWLWiVu+PPtYce66s6qZ/IjiyJk9Y141WvY5t3C99wN8DtyCKuRrnMaLG5ubjEAAkiyvb4yCWvaQdrXCx7WlMp9DQP+QGne3DzZeZKWm/axq7yipVLxdo3n1Jendgpml4HiWqgia9x5QyAYXLdWNz77rc23aoAkgbju3LLOLi8Mui01lDiSySp3lrjY4izgRsP5bdI8ulxA/V17YdYvjkbZ2UfYkfTXBvSXvmlhn2yMaT0OyePKBUkqZxRuJ0bHfY+UDq1yfWVc0gOXsBFiAQdhVG4WcWtPU3fF8DJjl4J6wr2hAHzNwi4IVdK4iSJxaPlsBc057slUqnAr7EewEWIBG44qJdwXoi8yGlhLz8osaT3pLYD5Lijc88xrndDQXHuClqPgvXS/F0dQeuNzR3vAC+r4aONgsyNjepoHoS6lkD5jouK3Ssn+GEd/1j2j6t1aNEcSNSJI3zVMTQ17HEMa5xOq7WsCSAFuiEgBCEIAEIQgAQhCABCEIAEIQgAQhCABeWXqEANa7R0UwtLG14/eAJHUcx2Kr6R4AxOxhkdGfFdz2+cgjvKuSFKM5R4ZFxT5KZwV4HvgqDUSva4tY5kbW3w1y0ue4kCxs0AAbysx4zeDLqWpe9rfgZnOexwyBdcvjO4g3sN3UbfQKa6R0fFPGYpmNex2bXC46D0HpCJScnljSSWEfKOopaOcEWGtdwA1bYXNgSMcbjAC21alpPieic4mCodGPEe0SAdAcCDbrupbgpxbQUsglkfy0jcW3bqsafG1bm5HSexRDBYOBuizTUcMLvCa27uhzyXOHYXEdimkBCBghCEACEIQAIQhAAhCEACEIQAIQhAAhCEACEIQAIQhAAhCEACEIQAIQhAAhCEACEIQAIQhAAhCEACEIQAIQhAAhCEACEIQB//9k=</t>
   </si>
   <si>
@@ -246,6 +243,9 @@
   </si>
   <si>
     <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/2wCEAAkGBxESEhUTEhIWFhISFRgVFRcWFRUWFxUWFRYWFxUVFRgYHSggGBolHRUVITEjJSkrLi4uFx8zODMtNygtLisBCgoKDg0OGhAQGy0lICUvLS0wLS0vMC0tMC0tLS8rLy0vLS01LS0tKy0vLS0tLi8tKy0vKy0tLS4tLS8tLS0tLf/AABEIAOEA4QMBEQACEQEDEQH/xAAcAAEAAQUBAQAAAAAAAAAAAAAABQECAwQGBwj/xABOEAABAwEEBgYFCQMKBAcAAAABAAIDEQQSITEFBkFRcZEHEyJhgaEyUrHB0RQjQnKCkrLh8ENiwhYkJTNUg5Oz0vEXU3O0CBU0Y2R04v/EABoBAQADAQEBAAAAAAAAAAAAAAABAgMEBQb/xAA6EQEAAgEBBQQGCQMEAwAAAAAAAQIDEQQFEiExE0FRYTJxkaHB8BQVIkJSgbHR4TNy8SM0YpJEsuL/2gAMAwEAAhEDEQA/APcUBAQEBAQEBAQEBAQEBAQEBAQKoaqVRGsKXgp0RxQoZAmiO0g6wJojtYVDk0Wi0SuULCAgICAgICAgICAgICClUCqBVEaqF4U6KzeIWGYKeFSc1YWm0hTwM52msLDagp4FJ2qFrrY3a4cwpjHPgztttI62j2sLtJRj6Y519ivGG/g57b02eOt49urC7S8frE+BV42a/g5rb72aPve6WGTTbBsd5D3q30W3fo5537j1+zW0+z92jPrVC3N0Y+tI0KewrHW0K/Wue3oYbT7f2R8+vMA/ax+F5/4U4MMdbH0reN/Rxaev/MNZmvULnACXM53CB41CmIwKXtvSI4tI9Uafy6Ky6bp6Y8W/BVzYOGNa9G+7d69rbs8nK3d4T5eU/qmrHbo5PRcD3bRxGa45h9LS2rZULiAgICCx0oG1TwyjVjNqarcEmqw21qns5RxQxu0gFbspRxrDpEKeyONhl0u1uZA4mitGCZ6KzkiGjLrXZm5zRj7bfit67BmnpWfYzttOOOsw15Nc7NslB4Bx9gWkbszfhZ223FH3mA64RHK8fs09tFf6tyd7C28sUePsZI9Zwcmu8aBROwTHewtvekdKy2WafccmDxdX3LOdjiO9z33xaelPf/CrtKSHcPA/FRGCsOO+8s0+DE62PP0vYrdnWO5yW2zNP3mMzOP0jzVuGPBz3zZJ62n2te1WhrGl7zRrRUkqZmKxqyrS+W0VjnMvO9K68yhxEZa1tcOyCad5O1cttot3PosG5cOkcUTMoabXS1HOY+AaPYFn29/F2V3Rs0fcj3z+rRm1mndnNIftu+KpOW097orsGGvSkeyGjLpYnMknvxVeJ0VwRHRhOkio4l+yhjdb3KNU9lC+z6RcCpiUWxRMPRdTdZwQIpD2cmuP0e493s4ZdmDN92z5jeu7NZ7XF1748fP1/r63W2xpb2waU2jCneq58Gn2q9G+6d69ppiyz9runx/n9Wawa1zMwcQ8bnZ/ez51XG+lidXW6H0xHaAbuDhm0503jeESkkBBq2u0XQtKV1VmdHmun+kdkUro2R37hulxeGtJGYGBrTKq9zFu2kUi2bJFdecR36e5xW2i02mKV10QFo6Tpj6McY4l7/ZRadhu+vpZZn1R/Eq8eeelUfP0i2s5OY36sf8AqJTj3bXutPz+Rw7RPhCPm13tjv27/AMb+EKPpuxV9HD7Z/ynsc09bo+bWS0O9KaU8ZXnyqo+tqR6GGsfPqg+izPW0sEVtvHtY124k+NV07LvmbX4ckREeXcyy7HERrXr5pSB69y3Pm82YZn6TZGaGpO4U95Xl7TtuLFbhnnPk0x7JkyRrHvVbrWxuUbjxIHxXnX3lSekNfqu09bLjr24ejC3xeT7AFyX2/XpC0bor32n2LP+IVq2NiHBjj7XFcttrvPg1jdGCPH2/wAKHX61n9oBwYwe5ZTtF/FP1Xg/D75bOjNZbbaZBFE573u2A0wGZJwAHeVEZbT3otu/DSNeGHQ6P1vML+ptQoW4XhiR34ekPNbUzacrPLz7s7SOPD7Pnog9c9bRKSyI/NNOGy8fW4blnly8XKOjs3du7so4r+lPu8nATSlxXO92tdGOqhYQEBAQEEpoWchwVqy589dYexxPvWKp2wH8BXpx/S/J8JaOHb9I/H8XlEumZoX9h5I3HEfkvMs+9wzydBoTXu45pcCxzTg5uI5buaq2ez6qa1QW5nYe3rWirmg7PWAONPZyqE+g866RtZfk8RYx1JZQQN7G5Ofx2Dv4L293bNWdc2X0K85857o+fi4s+SfRr1l4VaLRU/rJce17XbNkm9u/3R4NsWKKVisNcylcfaS14VOsKjjlOil4pxSaKVUaylfHIQrVvMKzDfi0k5opyO5epi3rlx4pxx+U+Hz7nLfZKWtxSmdXNHQ2iOUyEAj9o57gIqC96IIDnOxz3c4w1renHbnr3fPtMlprbhjk5MyYVJXlauvRgEkj/QFB6xoBzOHgmqVRBNskY47qj308lApFaDW68XXjYf1gg6LVPTDLNNekbWNzS00zGVDllhir0tpLm2nDOSsadymtWn/lVpdMG3W0DWgDY2uNPEqLTrK2HFNa/a6od0tfWPhT2qraI0WCu7bhllsOaJKH9FBWh7kC6d/l+aBc7/Ygrc7ygXB+iUFzW0yw4EhDTV1ehNcp4onwS/ORGN7Wmg6yPsmlKem0ba40qamlD0U2i0V4Z6PG2rc+LJljNj5WiYmfCefun3eXe5m0zXjVYS9akaQtaoXdt0ROI0rZ8cxKD3/MvOPIckH0Ug+eOlR5+WvqcKMpwuA05kr3s8zGwY4jvtOrhpGue3qhwTyvDtPN2woqpEBAQEBBUPIqAc8+9Wi9oiYieUomsTOste4ZHhuwZ0293u5qIjVLbtcjY+yAC4YE7G9zQtbRFOXeNaC2Y4tDgdlPYsRv6X0YerY4A3XtJiJ9IFvpRO35EjbgQpmJjqiJiUdZ5bzQduR4qEszAgvkbRzhndcRyKDM2EdZdxoWg82Xtneg1Y4qkCpxNPScgvoRgcxgUBBcDgcMyMccKVw3Y1HJBQ4gDcCKjM1JNT3404AIKufU1wx3AAeACAEGSN5aQ4Zg1HhigxTxhr3sGTHuaOAcbvlRBc1B2vRGf6Vs397/AJEiD6MQfPHSuP54/gz8C93aP9hj/ulxY/69vVDgnLw56uyFFCRAQEBAQUQbGgGVL3eqC7kPzK1wxrdekayi7aDex/R2qMtZiUzXSWaSMRxMe1zr7ibwOLaVcBj62Deawi2szCJjm6a2WwGxwADFtHcCJCOZHtXZl07Knq+Lgwa9tkjzj9HLQtuukbsa8jzI9y5nYzgoM1taesfT13bvWPcgzWZp61oJqbo5GOo8iEGCAVIFaVPIVxKCsr6ucRtcTzKDNY7I6V1GhXpSbM8mSKetvOgs0dWvfedgTdFaUrhXdj5Ba/6VfNz8Wa3T5/OVPk8EgDWPoQCAHCmbiSK7cSf0FMRiv05InLlx87xy+fBpWyN7Xm/W9vO3DDyosb0mk83VTJF41hgCouzQMvODa0BzO4DFzj3AAnwQa8kt9zn0pfe59Nwc4kDkQgvag7PomP8AStl4y/5EqD6PQfPXSyP5476rPwle7n/2GP8Aun9HFT+vPqcZYdHulJOTRiScABxXkVx6856Nr5eHlHVtXrM3BrXSEZkDDwV4tT7tdfexmMs85nT18lobZ5MBWN2yuSa47cpjSUcWbHznnHtaFqszo3XXf7rHJjmkurHkjJGsMKo0EBBRBI6nOb1xjdlIC37ww8xTxWuK2l2+zTHaRE9/JdrHoy60upRzTjxGa9LaMVb4NY6wz2u0488R3SgLXbHzBjSaiNoYKbAMtgXi1pFeiNUmy1VYxp9FgFeDe0Vta2sRHgxpThmZ8ZR1mBILtrnE/rzVGjM0oM0j7znOObiXYd5qguExvXtoAA4BoaPIIMV39YILmjYkRqiZ0jV0os5a1lnjNHyNvyv9WPOhOzAEldExz4e6HNHTinrb5j8u+SNrGMDmmOGFx7D5WufJNdqL7I243RUivfmtKzpGusVj1aywvFrTppNp8uUR+c8vnrqxWmzslaDejcK3WSx1DWuJJDJGOxZUk02Ekq1qVvGusT5xy0nzhSmW2O2nOO+az4eMTHKfNqCTrY3MeR1sOOJxIGYPBZx9qs0t1hvEdnkia+jZEtkBwBB4Yrldrt9WdT3Swuml7MTmOIGTpKA0FM2MqATXtOpSgFb3Ti2ebRxW6PC2/fFceSMOLnbWIme6P3lyFriumi55ezS2rE1Q0dl0UH+lrLxl/wC3lQfSKD5/6WGVtlN7I/4172SOLYKR/wA5/RwcXDmtPl8UDaYG1EFbsUTOttDvCob35gAbyvKvMTM69Ia1iYrH4p5/Pq6KSyNia0vf1Ae0OZFHG18tw+i+VzqBtRiBt3UV+Ph9KZjyj46sJx2v6FdfOZ0j8tOfz00YpYWTNqHh7Sboku3HxvPotlblR1MHDBXmK5K9dY98fwzre+G2kxp36a6xMd8xPl3xPNqMaZYnsd/WQ1I30GY8FlH2qzWesOiI7PLE16WRK5XaICCiDG4ljg9uYQdJLpuK1R0kq2QChcKdqnrDYVvGeeDhlplv2mk26whJLJGPpV8h4rFm0ppL3YZkcz+tn5KBvaOsMkr2xQsL3uwa0Zk+7ikRqra0VjWTSGjpIXlkjS14zGB257th5KZjRFMlbxrVqljvWPJqhdQRnHtGlTTLLZXDNBXqv3jzQZbFAOsbUnMfSPxV8XpwyzzpjtPknrewVtp20ZHmcGXmNPkKeK1iNYnXyZzMxaNO6J+DQ1wobVMLtRC7qY25gRxUjYANgoL2GZJ3rPN6ctMH9OvqNWIw572EUa+zzl+4dXE+VrvBzGlXwTpafUptFYmKz3xP+fclIIx8upT02MLuLoWl3mSrTP25ZxH+nTXxhGaJgq/LasfvS0y20q9n0WylkaP/AGz716dP6f5Pg9qnXbZn/lHweLaXPaXl2fe4OjSaqt3YdFR/payfWk/7eZB9KIPCOkpv8/ZX1Y/a9fQ/+DT++f8A1eXn9O39vxcraCCbTeydaY2v/wCn1hr4dlq8iI6euPg6MszHFMdeGdPX86InWWR7rVaXHF3XSAcGuLWDgGhoHcAsL68U6unHpwRw9NGfVtrj19cvksrnbg5oBjPHrLlOK0wTMTPq+MMdprE8PlPu0nVIsZ/PphsuvvcerN7zqpiftTPqVmv2aR89JcyueXWAKYjUZ47K4jAHDNb12e9omYjoznJWJ0mXQ6ous7OsFoN1rhdd2Guc5hBwYXA3caVpQrs2SsVpPj5+H7dWGaZmY8HMyNxNBhU04VwXnWjnOnR0xPLmwvslcdv62qOGU6g0e45knmfanDKOKGzHYSMgo0RxwmdVpjZ5w97SWFpa6mYBpiPEK1OUufaYjJTSPW6jStgdpO0h0UYYxrAytKCgJJcefHBaxjm88nDba67NTW/shD6y6pPsx9Zh9FwFK8RsPcoyYpq02PeNNojWOU98OUkjIKwepE6rKIldGSCDuNVNZ0nVW8Raswm7U4dYXO/qrSwBx3HCh8CF1TER16S4ota1YmPSr7/H91bZY2yEGVxjmAAL7jnxyhoo19WYtdQCuFDmrXxxf0tYnxiNYn2dJZ4s0440xxxV7o10mvlz6x4NzR9nihY+jnODxdlmLSwdXUF0MLXdoufQAk0wqNpIjhrjr+/LXyiPBftbZbc+Xl1089fH9Fmi7z3z2t4pg66P3n9ljRwHsWMcq6z3t7WibaR0r+vcntS9XL5vvHYbn+8fVHvWuDFxTrPR4m9d4xirwV9Kfd5/s6TWrS4iYYmekRQ0+i0jId5C2z5eGOGHm7p3fOW8ZsnTu858XmFos7XGtF58vs6V0gZo5m7zULvTeifUmkrLfIC1sd7qBteXNLC8/ugOcBvJrkMQ9eQeX9JGrZkAtEYJkiHaA+kwEmo/ebUnvFe5e/u7PS1Z2fJ6M9J8JedtWKZjir1+Dy7SEYEji7+qtDe0RsJxveBXNtGzzivNbRy6T8JUxZZy0i1fSr8zClosLZKGYPv0A62INe2UAUDnNJFH0pUjNZWwxf0onXxjTn648Vcea2PljmNPwzrEx5R5fo2ohHZ46BjgwkOd1lOttDmG8xl0YMiDgHHOpA3UVbUikaR/P5+ruhrS1slvte7pp4fn3/OmpZWuZFNO8/OTVa3vc81ceVeay7Oa185dEW47690cvz70F1BWXZy34mzZbLUrr2bZbZLxWOrHJlisaynLJGG4BfYYNmrgx8Efn5vFzZJvbWWZ+imSGo7O/Cq87aN3Y7zrXk0pttqRpPNng1XYc5D9381xzu+sd5bekx933/wkbPqXEc5HcgsrbLSGNt63/DHtS9k1Ks4zc8/d+Cwts9WFt6ZZ7oSEeqFl/f5t/wBKynZ6sZ3lm8mzHqrZR9E8/wAk7GrK28M898JWy2VkbbrG0Ht4rSKxEcnDlyWyTxWlbbbKyVhY8VafLvG4pNYtGkqY81sVuOvV51pTUia+erYHNrg68wVHAmoXJbZ7a8n0uHfGDhibW0nw0n9mo3UW0+oB9tvuKj6NfwXnfezR973Syt1DtG5g+1+Sn6LdnO/tm8Z9jfs2pk1wsf1ZbmO0ag93ZW+PDaI4bdHHl31g4uOmuvz5rY9U7QzBkjbu6pPkQr/Rbx6NtE/XGzZOcxz/ACj4srNTJZCDLKCBvqacAqzs2k63nVb64x1jSkae+filP5Ik3W3qRtxoGmpO0k7/AGKtsOs6zMM/ra3DpTHb58Utbi6CINhieTSjQ1jjTvOH+6tky1x10q5Nj3fm2vLOTNE6d+saa+UeTgbfo+1yOJMExqc+rf8ABeda2r7TFiikaQ1maCtP9nm/wn/BVbut1I1HfPJftMbmQRnFrgWmU+qAcbu8+A2kB7CxgAAAAAFABgABkAEFyDTtlmqFrS+ilo1eaac1Ec6R3V3OqfV1x1QWOOdygPZOdNi92m3YcmOIzRrMctfGPN5WbZMlbzfDOnkgv5BTsPYkDR3F4W1L7Bp6E+2f3c9suSZ/1OvnEfro2LJ0ePJvSPBPAknxKpfaNjr6OP3r07a8aVnl5R8ejatnR7JKRWZoa3BrRESAPvYnvVa7bssdcMTPnP8ADqrs+SI9Nib0YHbOP8D/APat9Y7PHTBX2/8Ayt2GT8c/P5szejVo/bO8I2j3lWpvatJ1pirHz6kTssz1tMs8fR+wfTkP3B7lM75vPdHvU+hV8ZbUWpLBtl+8z/Qs7b1vPh7J/dWd31nvn3fs3YdVWjY/xe33MWFt4Wnw9n8o+rcfn7Y/ZuxaCp9E+LvyWNtrme/3H1Xi8/a8405rhPZbZNZzdAifQdnGhAc2p4ELC20yzndWLz9pFr5KTSo+6FjO0WRG6cfh70gdcH09Lyb8FXt7+K31Th8PfKPt+u0rRg+nL4J29vFP1Tg/D+rJqVrRNarZHE95LXOAIy9iTnt4rV3VgiedYezjRrPUHJR2tvGfatG7sP4K/wDWP2XDRzPUbyCjtbeM+1eNgxR9yv8A1j9lwsLfVHIKOOfFeNkpHSseyF4sg3DkFHGvGz6dIPko3Dko4kzs+vVc2zAZBOJaMMx0XdQnEnsZ8V7IqKJlpXFoyKrUQEBAQUIQY3QAq0WmEaLfkrdynjk4YV+TN3JxyaQfJ27lHHJpCvUN3JxSaQr1LdycUmivVN3KOKTQ6sbk1lOivVjcmshcG5NR829OljbHpVzo3EunijkkBGDXBvVgA1xq2MHxUDiI3SDaOX5oNy/aSMCOX5oI+1WmbJ1OSDu+hGztdpCNz3kFt6gAGJumlTsQfSiAgICAgICAgICAgICAgICAgtkkDQXOIDWgkkmgAGJJJyCDh9NdJ1liqIG9e4bb4jjJ+uQT4hpCDnH9LVq2WSzDjaXn2RBBb/xYtn9msv8AjyH+BBQ9K1s/5NlH95IfcEFh6VLd/wAux85T70Fp6U9IerYuUx/jQcBrRHNb7S60zWiIPfQUY0hrQ0AANBJOQ2lBHDQH/wApv3UGQaEP9tPhX4oMTtXGHO114gn3oJXVyI2GVssNpYXNNQHsJFfBwKDqZOme3xvuyQwHaC0Oo4bwaoJXR/TFI/0omDhX4oOnsPSAJBkAgkRraO5A/laO5BT+Vw7kFP5XjuQbNk1uiJAk7NfpDIcRsCDo2kEVGIOSCqAgICAgICAg8T6c9anulFgicRHGGvtFD6T3dqON3cG0dTbebuQeT3jvQLx3oF470C8d6BeO9AvHegXjvQUvHegVO9Aqd6BUoLXtvU7jUe8ePwQTVisNKFBOWWS7tQbgtx3oLvlp3oKi2HeguFsO9BcLWd6D0Lo41mY8fJJH/Otq6IGtXMxJaDlVtCaZ07gg7xAQEBAQEBAQfKmvFpMmkbY45/KZWeEbzG3yYEEKgICAgICAgICAgIANMdyCeZNdFNgJA4AkBBU25ozcOaC06VjH0xzQWO03EPpcgT7AgxnWKPZePgUGJ+s4GTHHl8UGSy60ioDoSSSAO1TM0xQSmh9IOZa4Jxg5s0Zw9W+AW8KEjxO9B9OICAgICAgICD5O1r/9fbP/ALlp/wA+RBFoCAgICAgICAgICChQZNZCQBT13e0oIHrHbzzKB1jt55lA6x288ygdY7eeZQOsdvPMoNnR8MksjWNcak1rU9kDMoO90Do0yWyzWdgJvSx51JuNIc812mjXHwKD6aQEBAQEBAQEHzF0naMNn0naWkUbK/r2H1mzdokfb6xv2Sg5dAQEBAQEBAQEBAQVjZeIaMyQOeCCzWWTFo3lz/Ans+9BBoCAgIKoO21b0WY2io+dkpXuGxvx/JB73qDqsyzsbO9o69zSATm1rqE86D9FB2KAgICAgICAg4/pG1HZpOJt1wZaYa9U8+iQaXo5KY3TQYjEHHHEEPC9I6j6TgcWvsUzsc4o3TNPeDGDhxog0jq5bhnY7SOMEo9rUGF+hbUM7NMOMT/ggwSWKVvpRvHFrh7kGBwpnhxwQUBQXXTuKClEBBRBVBa61tiOOLt27fXv+KCKtlpdI8vdmfIDIBBgQEBAQTmrejr7uscOyw9nvd+XwQey9GurfXSddIPm2Y8TsCD2IBAQEBAQEBAQEBAQEBAQULRuQef69a4wQNLImsc81F4BpJO0Mw5u2bMUHi9ttJlcXODe4AAADcEGo+m4ckGnNJuPmg0ZZ3bHO+8UGtJaX+u7mUGoUFEBAQEGxYbKZXhg25ncNpQekas6GM0jIY24YD/dB9C6G0ayzxNiaPRGJ3naUG8gICAgICAgICAgICAgte8AEkgACpJwAAzJKDzHX7pADQYYDngTkXDv2tZ5u7hVB5HabQ6Rxc81cf1QbggwOcgwSvQaMzkGnIUGu5BicgtQEBBUIOv0Fo7q2jD5x+fduag986NNWxBF1zx848Ydw3oO3QEBAQEBAQEBAQEBAQEHm3Tbb7RDBAYpRHG972vFAb7rodGOAuvNOG5B4JNbrRWrrricSaONTvzQYjpOTaweaC06Ud6nn+SCx2ka/R80GF1rB2FBidKO9BjJQWEILaIFEANQTGr9hvO6x2TT2Rvdv8EHrPRtq0bTMJHj5tmJ7+5B7g1oAAGQwCCqAgICAgICAgICAgICDDa7SyJhfI4NY0VJP6xPcg8e6RtKfL20Auxw1Md7HE4Fzhvph3VKDyaeOUEtAaS3Ps0p3ccsO8IML2TDOMcj8UGsbQ6paQAQO/4oNb5Q+uzkEGQPdubyQK/ut5IFR6g80FrnMGbfNBbfj3HmgVj7/JBVtwZOIPBB1eplifaHCNhLqvplvAwQfTOrmiG2WBsTRiBVx3lBJoCAgICAgICAgICAgICD581r6TxapS10UrI43FrWtc0Yg0JeD9LZ3bN5CEdrZZyKEzAHYWNIQY//ADqynKUj68Zqgvh0nZa1M0Z3YXedSgvltFmdkWH7pQR1pskJyY3waPcgirTZWjIEcwgjpARkUGB0rht8ggxveTmgtqgVQZLPE57gxoq5xoEH0n0Q6ots0Imc3tEdmufe5B6SgICAgICAgICAgICAgICD5W6U9FfJtKWpgFGyP65nCYXzTuvl48EHKICAgoWjcgBo2BBeHu2OcODnD3oLhaH+u7xJPtQWmVxzoeLGH+FAv/us+4B7KILaN2xt8L4/iQCGepTvDifI5oPQeiDVdtptUl5vZiayp2UcSSePYp4oPpCKMNAa0UAFANwCC9AQEBAQEBAQEBAQEBAQEHif/iI0K69Z7Y1tWhroJXD6ON6K9uFXSCu8gbUHi4KAgICAgICCiAgICD1voA0zctMlnccLRF2f+pZ6kAcY3k/YQe9ICAgICAgICAgICAgICAgILJY2uBa4BzSKEEAgjcQc0EJadS9GSelYLMf7iMHmAgi7T0W6GfnYmt+o+Vn4XAIIu09C2iXeiJ2fVmJ/GHIIu0dBFjPoWu0N+sIn+xoQRVo6BX/s7e0/Ws5HmJPcgi7T0G6RHoT2Z/EysP4Cgi7V0P6YZlDHJ9SZn8d1BFWjo50uzOwSn6pjf+FxQRdp1at8fp2K0t4wS053aIIyVhaaOBaRscC08igsDhvCCf1FtUsdus7oWl0jZo3NaM3doMe37THuCD63QEBAQEBAQEBAQEBAQEBAQEBAQEBAQEBAQEFr4w7AgEd4qgjrVq9Ypf6yyQP+tDG72hBg0fqlo+CQSw2SGOQZOZG1pFQQSKZGhIr3lBNICAgICAgICAgICAgICAgICAgICAgICAgICAgICAgICAgICAgICD//2Q==</t>
+  </si>
+  <si>
+    <t>data:image/jpeg;base64,/9j/4AAQSkZJRgABAQAAAQABAAD/2wCEAAkGBxETEhMQEhISFhUVFxUZGBUVGRgdFxgYGBkXHRcXFRUYHSghGBslHBUYITMiJSkrMC4uGh8/ODMsNygtLysBCgoKDg0OGxAQGi0mICEtMjcuKzc3LSs3LjIuMy8uNjEtKy0tNy0tLystMi83Ny0uLS0tMS8vLSsxLS0tNy43Lf/AABEIAN0A5AMBIgACEQEDEQH/xAAcAAEAAgMBAQEAAAAAAAAAAAAABgcEBQgDAgH/xABAEAACAQMCAggDAwoGAgMAAAABAgADBBESIQUxBgcTIkFRYXEygZEUocEjM0JScoKSsdHwCENiorLhFfEkRIP/xAAZAQEAAwEBAAAAAAAAAAAAAAAAAwQFAQL/xAAuEQEAAgECAwYFBAMAAAAAAAAAAQIDBBEhMUESUWFxkaEFEyKBwUKx4fAUMtH/2gAMAwEAAhEDEQA/ALxiIgIiICIiAiIgIiICIiAiIgInxVrKoyzKo8yQB98xRxe2JwK9HPl2iZ+mYGbE/AZ+wEREBERAREQEREBERAREQEREBERAREQEREBERAREQEgPWb0ye1AtrdgKzrqapgHskOQukHYuxBxnIAU5HKTi9ukpU3q1GCpTVnZjyCqCWJ9gJzJ0l441evVrvs1Vi5B/RB2RP3UCj3zOxA+7GhVvLqlTLu9Sq4U1ahZ2UE95ueSAATjI5eE9ekPBriyKHL4cHvhXUagzqVBJ3BCagdiQeQkh4Le0bay/8lSp0XZqaUKhqXLpUD0xTVqVKlTp5Ovs1qfHuG8AMST3HSihd8FrXNxTVQddIU85Bqj812bEZz8LZxthuYE6K96MdNLqzrUmNU9kWAdW+BgdjqHgRnOob7eI2PRdhdrVprVXkwz7eBB9QQR8pyvXph6bL44/lLb6leknaUhb1D3hld/1kGR/FTH1pt5zu0bIb3ml678p4ffp68vPZasRE8JiIiAiIgIiICIiAiIgIiICIiAiIgIiICIiAiJDen3TulYoaaFXuCuQp+GmDyer+C8z6DeBoOunpSlOkLFW3bS9bB5IDlKZ9WYA48l32ac+V70sxY8zNpfdIHe4NUuWLkl2OO+W55HIj05TYHhVtU76aKbkYKsCUOcd5P1TgeIPP6dEcW5Jx/Y8M/yE2F5xWuyU6RBFKlkIig6FLbsx83bcknfywAAJ5xOlwgWFWhRtH+1siharsrKHyNZRjULKMatsSM8NUJcU6lVKdSilTU1Fj3XBCBgRuMkJz9swNLacWwcGS3oZfmhcrUpnC1MEHw1A5TPmA3dPoxmo6WcRtWqdpStaVEfo0kLMB6sWOPoFHLaafg9+xra2YlsYGTt7egiePBFmx/MpNffunpP2l2Bw+8WrTSqvJhn2PIg+oOR8pkyrurfpUuRRqHu1CME+D7AZ99h748zLRkeO/ajjzjm5gyTev1RtaOceP/J6ERE9piIiAiIgIiICIiAiIgIiICIiAiIgIiIGi6a8d+x2lSuoBf4aYPLW3InzCjLEeIWcpcc4u9Z3Jdm1MSzE7ux5kmdI9b9i9WwZUBLb4A89JP4EfOctuuJ3ojpk3vavd+f7L45kYkttbmkKSK53Cj3kUo88+W/9/OGZicb58v8AqInZIvno10ss0FrTNyiaLZO81TCqRWUvTIOyvoXffLDA8BND1h9IrapaUBQuKblamdAPeCMtXQSvNdAGjHhqErC3FwEZQcKRnBx3g+BsOZzpH0HpPqva1nPeYEguPUHOps4Hm2fnAxbyqWYkzyoneela3ZfI5AOQfAzyXnOCY8A4mV0OfB0VvUE4z9MzpXonxE17cFjl0JRz5lQCCfUqyk+pnMnRKxatVo0QM6qqMfRKfeYn0wCPcidFdAaTKtznl2qgepFKmSR/Fj92VLZdtVFI613n14flWmZ/yIiOU1nf1jb8pXERLayREQEREBERAREQEREBERAREQEREBERAxeKWYrUnpH9IbHyYbqfkQDOZesfgHZsblV05YpVT9WoCQSPQkH5+86klUdavDAftIA2q0RU/wD0XIz6fBTP1lTV3tj7OSOUTET5Tw9mdronFamor0mInxrM7e08lB8I2qZzjCsR74xv9ZndmorBcgKOZHjhc/XO8weFt+UIAyWUqAeWT5zMa3zWVM7DVk+eld/r+Muw0WR2rY7YsNYCBRjnk88f6sbT6ZyvJgWqa9XkuOWT5Ljf5+kJVJxXZVwuhQPDxy3y8PnPnDKMFQWqhsDyydh88b/9Toxbuj3lohgVyoz6uRqJ/nPG95jlhdSj1wc8/E77/wDc9rqiQwp/pAoC3me7v8uXymw4PYrXu7aiRhNXeXngKSzhs+Jx/uHnI8l4pWbTyiN3qtZtaKx1Wp1bdHUtLQ3tcYd0zjG6UuYAHizHBwOfdHhLV4HZdjRVD8R1M/7bks4B8gWIHoBK+q3Zr3ljZL8LVe2qY8KduNYHsagpj6y0ZifB8eTJN9Xl/wBrzw8Ij++yXU4oxX7PXqRETcQEREBERAREQEREBERAREQEREBERAREQEgPWiAKNxVP+Xav/v1gfeJPjKY64+OgWt0it+dqpSH7KY1D2yjn96Z/xGZmlccfqtWPfefaHqMHzYneOEcfT+VG2mdeFGScqPc7AzKqp+VC5O3aZPicA5x5ZAP1mFZk9ounOc7Y8zsJl133QZwctqYc8HA/ln6zReWxDIWFbQRTU0wB6hTg+oGMTzyFRtQbW6dweQLbAepP4T0TQzYJPYqyhR4Fgo29vE+4855iqSvas51gAIN8kFvi9c8hPQxL8FTzOsMMn/Vvy9Bt9JIuiTqtxrB7qUsAnnlj3ifXnI5f1WGSSMlt/cb4+RGPlN/wRBmppOQNK6v1jjJP1Y/LEraqs2xWrHVqfBsMZdbjrPn6RMrO6q2Nfi9zWzkULVaYHhmo6tn6KR/6lxykOo/jdrSrX6Vq1KnUq1KKoKjBS+O0UKmT3jkjYeYl3zuDHGPHWsdIVNZft6i9o75/ciIkqsREQEREBERAREQEREBERAREQPxmABJIAHMmaC56bcNQlWvKGRz0tqx+0Uzj5zXdY/RC44ilGlSu+wRGY1EKalq506dQ1D4cHY5B1eglR9ZXVu1haLXNxWrkMAxFNKdBATgdwOSCcjGAeRzjaBcJ6yeDj/79D6t/SSHhfE6FxTFa3qpVpnYMjAjI5jI5H0nO3Ud0UtL+rcfaqZcURSKrnCnUXzqxufhHj5zoPgfA7azpmla0UpIWLFVzuxAGTnmcAfSB98c4gLe3rVz/AJaMw9SB3R8zgfOcr9OeKtV7KmSTpyxz4k7An6H6zoHrYuCtmtMf5tVAfZQz/wDJVnMXSCpm4qejY/h2/CR3wTa9ck8o3282rSsYvh1r9cloj7Rx/d+cJtyXVgdOCTq8sAnl68vnNn/4xSB38eOQBnljx8MeEw+FX1NQFcY9ZuUq0GGQZNEMp8CwDKtMuAqnIGPrvn756jhbF1qa6R0hQAVIAx44z/e0+T2f60/FYHYN/eJ3YeF1wthSqVXYaDk6gBq57YBbYEge+3KbHopTBpMRkgt4+iqD9+flNDf3oJFIsezyM+w/lMhboKuaVOoyg8wuEH7wJz909UtFbbzG7Q+Gav8Axc/zZrvtEsK1XVeIucZrKM+9Qf1nZs41pcQd3VTVNNSygsuQFBIBbY5IGc4z4Tq7odwSrZ2wt6t1UuWDMe1qAg4PJQGZjge5kShad5mW8iIhwiIgIiICIiAiIgIiICIiAiIgJC+uK17ThF0oGSOyb5LVplseunMmkr/rp4yaFitIc69QKf2VGo/eFHsTJ9Ngtny1xV52l2Nt+KqOrDpKODmvVuKZYV1QKqkahoLHJHl3pZ3AOujhtw/Z1e0tiTgNVx2Z93UnT+8APWULxWhVrFWRSQF55Hj7mYi8ErHB7oz5k/gDO6rHXHmtjr+mdvR6ydjtfRydN9Z9NHsRX1rppvTfVnYq2U7p5HeoD8pzP0osyldmA7rnUD4b8x75zNta1b+nQazW5PYsQxoHJQ4OrKhhsc74GMkDMwCtcKUYq6+TDOD7bET1TLScU4r9+8T+J8JWa6iJ0/yL9J3ie7w8paCfSuRyM2NzYqQuhWU47xZwwY+a4RdI57En3238VsDnfl5cj94lVTY/2hv1j9Z+iu3PJnsLBsHz8Bj658R9JkWlmF3cZPgPD3P9JZ0mly6rLGLHHGfbxlyZiObBWi7bhWPsDJFw+qRZshBHe5H9pTMG74iR3V2PiR4egmELt9LZJOSOfv8A9S9aNNpL2pW82nszEztw3mOnfxWcWWMe+3WJj1eVIbH+/AzsXoldtWsbOs3xVLeg592pqT/Oce24JGwydsAeJ3wJ2N0asTQtLa3POlRpUz7oig/eJkK7ZREQEREBERAREQEREBERAREQEREBK366eG9rRtT4Cqy/NkJH/AyyJrOknCFurd6BJUnBVhzV1IZG9gwGR4jI8ZY0uecGauWOko81Jvjmtecw5mNVVP5zTjIwfDBO3tknE+xVIznSc42/SOfIevlPLpb0R4hbXNVHt6j76+0oJUakQ3eyrafAkjfymkqWF4hBahcKSNs03G3iRkesivbtWmXqu+0b80gatsNS+x5nPt+EO42JXBP3j1kYd61M5YVFJyO8CPfGZ5rxBxnvHf8AvE88HpKSEzjQd+a/jk8p8fkhtjbyPh7H6/3yjX298Y1f34T4qXTEacxwGzp5uK4pU86Bz35gfEfbO0zOPYogIvxt9w8/wmR0Nq0LehWuqzAFiERNtbaRk6V9SQM8tpi2fCbziNVqlG3q1C3LQp0Ko2ALnCj5keM1cWqjTaSa0n678/CGfE3zameH0U95/hHws+KzfoiTvhnVxeI7G8tr2milfzFBa5YHn8NUYxtyDc+W0+On/Rvh9tQSpbHiIqmoFdbug1NSpVyWUmmoDAhRjPL2MyWg1/Vhw2rX4japSyCKquzAZ0pT7zncYG2wz4ss60lK/wCGuspp3tPSupXpNqx3irhhgnyBTl6mXVAREQEREBERAREQEREBERAREQEREBERAREQIF1pdAKvFRR0XIpdjr7jKSrF9PeJBBBAXHI8/DfMxHC6OAGpUm2AyUU528ciZkQIp0j6NcMp21xcHh9mTSpVan5ilk6ELeQ8vOcq17dQ5CkkAZ39s4++do3FBHVqbqrIwKsrAFWUjBVgdiCDjE5t65uAWtle0qdrS7NXoh2UM5Gou421MdIwo2GAMQJF1B8LtbmlcrcWlrVNFqRV6lNWf8oHyGLZBA0DGw5nnLyp0woCqAAOQGwHsBylG/4fX03d5TDEA0kbTk76XxnHjjVjP+r1l6QE13HOB215T7G6pLVQMGCtnZgCAwIOQcMR85sYgabo70VsrEOLSgtLXjVgsS2nOMliTtqP1m5iICIiAiIgIiICIiAiIgIiICIiAiIgIiICJ51q6oNTsqgeLEAfUyOcR6wuE0c6763OPCm3aH2xT1HMDacS6QWluwp17ijTYjOl2AON8HHgNj9DMY9MuGeN/ZD3r0h/Npz91g9JqVzfVbi0uLgpUCd3SyadKIvdy+TnST8K4z47mRv7dV8AxPm3j6kY/GB1bR6R2LgMl3asDyK1qZB+YaUN193iVOI0jTdXUW1MakYEZ7SrkZHjy+sgtxeVsbuF9AB/Q/zmCC7aixJwpIJ/D6QLN6k+I0qPEa9StVp0qf2aplqjKq57WhgamIGecul+m3CxueIWXyr0j/JpyczMFyGYNhTkE5IIGQT/AHynmL2p46T7qu/zAB++B1bU6wuErzv7Y/svqP0XMyuDdMbC6qdjb3CVKmktpAYHAxkjUBnGROSlvB40/wCFiP8Alqkj6BdJ7exvKd3UWuQgbuU9H6SspBLEahhs+G4EDq+JBeH9bvB6uAbk0yfCrTdfqwBX75JOHdJ7GucUbu2qH9VKqFv4c5gbaJ+Az9gIiICIiAiIgIiICIiAiIgIiICRPrUvq1Hhd1UoOyVAKYDISGANRA5UjcEIWOfDElkobr8uX+20qTboKCsmeQLPUD4yPi7i5Plp5Y3CO8C6E3nFVe4Ru0Ctp11ahwW5kKTknGfwklsepS7xpd7RBkHANRzn11Uxj5HEkP8Ah6YfY7kBSMXHxeB/JU+R9NvqJasClL3qaulC9jXoOSwDBg1MKv6wI1avbAm54T1L2wXNzcVnffIpaUpjyxqVmJ9cj2EtKIEDo9UHBx8VCo/7VaqP+DCQvrk6G2Npb0alrQFJnZ6baWfBHZuwyrEj9A785eEqj/EBeUvstCl21MVlrK/Zah2hplKiFgnPGTz25HnA1PU90OsrmlXqXVBKpVqaKWJ2XskYjSDjOWO+Mya3HVLwVsn7JpJ/Uq1h9F14H0mu6hbNk4dUqHGK1xUZfPChKeG8u9Tb5ESyYFbV+pPhLcvtKfs1eX8SmaDiHULTNRewvXWljvCqivUz5qV0jB25jb15S6IgUfV6gW/R4gD+1b/0qyIdOerWtwynTrvcUagZwqqoZWzjOQDnPKdPyqf8Qw/+Ja5XI+0Yz4D8nUx89j9DAkXU/VB4VbLrRigcEKwYqC7FVfHwsFIyp5SaShuoOtUN7WQZ0C37xHLZ0FNW8zu+M77N4cr5gIiICIiAiIgIiICIiAiIgIiICabpJ0Ws74It1RFTQSVOplZc88OhBwcDbONh5TcxAwuD8JoWtJaFvTWnTXkozzPMkndifEkkmZsRAREQE5m62TUHE7tKmrGpGXI+JCiFfHcDdR4d0+OZ0zNfxPgdrcFWuLehVKfCatNWK+xYbQIx1M02XhNvqUrk1mGfFWquVbHkQRjzGD4ybz8VQBgDAHgJ+wEREBMbiPD6Nem1GvTSpTcYZHGQfLb33zMmIGs4HwC1tFKW1FKQY5bSN2I5amO7fMzZxEBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERAREQEREBERA//2Q==</t>
   </si>
 </sst>
 </file>
@@ -342,10 +342,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -715,7 +711,7 @@
         <v>28</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -723,7 +719,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -731,7 +727,7 @@
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -739,7 +735,7 @@
         <v>27</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -747,7 +743,7 @@
         <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -755,7 +751,7 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -763,7 +759,7 @@
         <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
@@ -771,7 +767,7 @@
         <v>25</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -779,7 +775,7 @@
         <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -795,7 +791,7 @@
         <v>4</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -811,7 +807,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -819,7 +815,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -827,7 +823,7 @@
         <v>8</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -835,7 +831,7 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -843,7 +839,7 @@
         <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -851,7 +847,7 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -859,7 +855,7 @@
         <v>34</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
@@ -867,7 +863,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
@@ -875,7 +871,7 @@
         <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
@@ -883,7 +879,7 @@
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
@@ -891,7 +887,7 @@
         <v>11</v>
       </c>
       <c r="B26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
@@ -899,7 +895,7 @@
         <v>3</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
@@ -907,7 +903,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
@@ -915,7 +911,7 @@
         <v>23</v>
       </c>
       <c r="B29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
@@ -923,7 +919,7 @@
         <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
@@ -931,7 +927,7 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
@@ -939,7 +935,7 @@
         <v>7</v>
       </c>
       <c r="B32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
@@ -947,7 +943,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
@@ -955,7 +951,7 @@
         <v>13</v>
       </c>
       <c r="B34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
@@ -963,7 +959,7 @@
         <v>20</v>
       </c>
       <c r="B35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>